<commit_message>
Updated stealth tactic rules for multiple log sources
</commit_message>
<xml_diff>
--- a/ocsf_mapped_new_sprint.xlsx
+++ b/ocsf_mapped_new_sprint.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O376"/>
+  <dimension ref="A1:O382"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26780,6 +26780,468 @@
       </c>
       <c r="O376" t="inlineStr"/>
     </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>AN0071</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>stealth</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>T1218.015</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>Electron Applications</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>DET0025</t>
+        </is>
+      </c>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>Electron Application Abuse for Proxy Execution</t>
+        </is>
+      </c>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>host-local feeds only</t>
+        </is>
+      </c>
+      <c r="J377" t="inlineStr">
+        <is>
+          <t>WinEventLog:Security; WinEventLog:Sysmon</t>
+        </is>
+      </c>
+      <c r="K377" t="inlineStr">
+        <is>
+          <t>Detects abuse of trusted Electron applications (Teams, Slack, VS Code, Discord) via malicious command-line flags (--gpu-launcher, --inspect) or spawning of unexpected child shell processes.</t>
+        </is>
+      </c>
+      <c r="L377" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M377" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N377" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O377" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>AN0091</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>stealth</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>T1564.001</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>Hidden Files and Directories</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>DET0032</t>
+        </is>
+      </c>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>Hidden File or Directory Attribute Setting</t>
+        </is>
+      </c>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>host-local feeds only</t>
+        </is>
+      </c>
+      <c r="J378" t="inlineStr">
+        <is>
+          <t>WinEventLog:Security; WinEventLog:Sysmon</t>
+        </is>
+      </c>
+      <c r="K378" t="inlineStr">
+        <is>
+          <t>Detects adversarial use of attrib.exe or PowerShell to set hidden and system attributes on files or directories, concealing malicious artifacts from user and administrator inspection.</t>
+        </is>
+      </c>
+      <c r="L378" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M378" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N378" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O378" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>AN0113</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>stealth</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>T1070.009</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>Clear Persistence</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>DET0040</t>
+        </is>
+      </c>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>Persistence Artifact Removal for Anti-Forensics</t>
+        </is>
+      </c>
+      <c r="I379" t="inlineStr">
+        <is>
+          <t>host-local feeds only</t>
+        </is>
+      </c>
+      <c r="J379" t="inlineStr">
+        <is>
+          <t>WinEventLog:Security; WinEventLog:Sysmon</t>
+        </is>
+      </c>
+      <c r="K379" t="inlineStr">
+        <is>
+          <t>Detects adversary activity removing persistence artifacts such as scheduled tasks, services, or registry run keys using sc delete, schtasks /delete, or reg delete — indicative of anti-forensic cleanup.</t>
+        </is>
+      </c>
+      <c r="L379" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M379" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N379" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O379" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>AN0118</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>stealth</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>T1218.012</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>Verclsid</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>DET0042</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>Verclsid LOLBin Abuse for COM Object Execution</t>
+        </is>
+      </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>host-local feeds only</t>
+        </is>
+      </c>
+      <c r="J380" t="inlineStr">
+        <is>
+          <t>WinEventLog:Security; WinEventLog:Sysmon</t>
+        </is>
+      </c>
+      <c r="K380" t="inlineStr">
+        <is>
+          <t>Detects abuse of verclsid.exe (a signed Windows Shell binary) to execute arbitrary COM objects via CLSID arguments, which may load malicious scriptlets or DLLs.</t>
+        </is>
+      </c>
+      <c r="L380" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M380" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N380" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O380" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>AN0139</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>stealth</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>T1564.012</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>File/Path Exclusions</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>DET0051</t>
+        </is>
+      </c>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>AV Exclusion Path Addition or Abuse</t>
+        </is>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>host-local feeds only</t>
+        </is>
+      </c>
+      <c r="J381" t="inlineStr">
+        <is>
+          <t>WinEventLog:Security; WinEventLog:Sysmon</t>
+        </is>
+      </c>
+      <c r="K381" t="inlineStr">
+        <is>
+          <t>Detects adversarial modification of Windows Defender exclusion lists via PowerShell Add-MpPreference, or execution of binaries from paths commonly excluded from AV scanning (e.g., C:\Windows\Temp, Exchange directories).</t>
+        </is>
+      </c>
+      <c r="L381" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M381" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N381" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O381" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>AN0182</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>stealth</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>T1564.011</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>Ignore Process Interrupts</t>
+        </is>
+      </c>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t>DET0067</t>
+        </is>
+      </c>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>PowerShell Silent Error Suppression for Evasion</t>
+        </is>
+      </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t>host-local feeds only</t>
+        </is>
+      </c>
+      <c r="J382" t="inlineStr">
+        <is>
+          <t>WinEventLog:PowerShell; WinEventLog:Security; WinEventLog:Sysmon</t>
+        </is>
+      </c>
+      <c r="K382" t="inlineStr">
+        <is>
+          <t>Detects PowerShell execution with error action preference set to SilentlyContinue or Ignore, used by adversaries to suppress error output and execute commands without alerting users or detection tools.</t>
+        </is>
+      </c>
+      <c r="L382" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M382" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N382" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O382" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refactored discovery rules to support multi-logsource splits and updated tracker
</commit_message>
<xml_diff>
--- a/ocsf_mapped_new_sprint.xlsx
+++ b/ocsf_mapped_new_sprint.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O382"/>
+  <dimension ref="A1:O390"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27242,6 +27242,622 @@
         </is>
       </c>
     </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>AN0016</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>T1482</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>Domain Trust Discovery</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>DET0007</t>
+        </is>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>Domain Trust Discovery via nltest and PowerShell</t>
+        </is>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>host-local feeds only</t>
+        </is>
+      </c>
+      <c r="J383" t="inlineStr">
+        <is>
+          <t>WinEventLog:Security; WinEventLog:Sysmon</t>
+        </is>
+      </c>
+      <c r="K383" t="inlineStr">
+        <is>
+          <t>Detects adversarial execution of nltest.exe, dsquery.exe, or PowerShell AD cmdlets used to enumerate Active Directory domain trust relationships.</t>
+        </is>
+      </c>
+      <c r="L383" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M383" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N383" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O383" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>AN0037</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>T1217</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>Browser Information Discovery</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>DET0013</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>Browser Artifact Access for Reconnaissance</t>
+        </is>
+      </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>host-local feeds only</t>
+        </is>
+      </c>
+      <c r="J384" t="inlineStr">
+        <is>
+          <t>WinEventLog:Security; WinEventLog:Sysmon</t>
+        </is>
+      </c>
+      <c r="K384" t="inlineStr">
+        <is>
+          <t>Detects non-browser processes accessing local browser profile artifact directories (Chrome, Edge, Firefox) which may indicate browser information discovery for credential theft or reconnaissance.</t>
+        </is>
+      </c>
+      <c r="L384" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M384" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N384" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O384" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>AN0048</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>T1518.001</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>Security Software Discovery</t>
+        </is>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>DET0016</t>
+        </is>
+      </c>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t>Security Software Discovery via Service and WMI Queries</t>
+        </is>
+      </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>host-local feeds only</t>
+        </is>
+      </c>
+      <c r="J385" t="inlineStr">
+        <is>
+          <t>WinEventLog:Security; WinEventLog:Sysmon</t>
+        </is>
+      </c>
+      <c r="K385" t="inlineStr">
+        <is>
+          <t>Detects adversarial enumeration of installed security products (antivirus, EDR, firewall) using sc.exe query, wmic product, netsh advfirewall, or PowerShell WMI queries.</t>
+        </is>
+      </c>
+      <c r="L385" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M385" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N385" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O385" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>AN0095</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>T1057</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>Process Discovery</t>
+        </is>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>DET0034</t>
+        </is>
+      </c>
+      <c r="H386" t="inlineStr">
+        <is>
+          <t>Process Discovery via Enumeration Utilities</t>
+        </is>
+      </c>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t>host-local feeds only</t>
+        </is>
+      </c>
+      <c r="J386" t="inlineStr">
+        <is>
+          <t>WinEventLog:Security; WinEventLog:Sysmon</t>
+        </is>
+      </c>
+      <c r="K386" t="inlineStr">
+        <is>
+          <t>Detects adversarial execution of process enumeration tools (tasklist.exe, wmic process, Get-Process) used to discover running processes on a compromised host.</t>
+        </is>
+      </c>
+      <c r="L386" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M386" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N386" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O386" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>AN0240</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>T1518.002</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>Backup Software Discovery</t>
+        </is>
+      </c>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>DET0088</t>
+        </is>
+      </c>
+      <c r="H387" t="inlineStr">
+        <is>
+          <t>Backup Software Discovery via CLI and Registry</t>
+        </is>
+      </c>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>host-local feeds only</t>
+        </is>
+      </c>
+      <c r="J387" t="inlineStr">
+        <is>
+          <t>WinEventLog:Security; WinEventLog:Sysmon</t>
+        </is>
+      </c>
+      <c r="K387" t="inlineStr">
+        <is>
+          <t>Detects adversarial enumeration of installed backup software using service queries, registry reads, or WMI commands targeting known backup product names (Veeam, Acronis, Windows Backup, ShadowProtect).</t>
+        </is>
+      </c>
+      <c r="L387" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M387" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N387" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O387" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>AN0254</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>T1033</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>System Owner/User Discovery</t>
+        </is>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>DET0093</t>
+        </is>
+      </c>
+      <c r="H388" t="inlineStr">
+        <is>
+          <t>System Owner/User Discovery via Command Line</t>
+        </is>
+      </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>host-local feeds only</t>
+        </is>
+      </c>
+      <c r="J388" t="inlineStr">
+        <is>
+          <t>WinEventLog:Security; WinEventLog:Sysmon</t>
+        </is>
+      </c>
+      <c r="K388" t="inlineStr">
+        <is>
+          <t>Detects adversarial execution of commands to discover the current logged-on user, system owner, or local network groups (whoami, net config, net user, net localgroup).</t>
+        </is>
+      </c>
+      <c r="L388" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M388" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N388" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O388" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>AN0271</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>T1010</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>Application Window Discovery</t>
+        </is>
+      </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>DET0097</t>
+        </is>
+      </c>
+      <c r="H389" t="inlineStr">
+        <is>
+          <t>Application Window Enumeration via Scripting Host</t>
+        </is>
+      </c>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>host-local feeds only</t>
+        </is>
+      </c>
+      <c r="J389" t="inlineStr">
+        <is>
+          <t>WinEventLog:Security; WinEventLog:Sysmon</t>
+        </is>
+      </c>
+      <c r="K389" t="inlineStr">
+        <is>
+          <t>Detects processes using PowerShell or scripting utilities to enumerate open application windows via Win32 API calls or cmdlets, which may indicate reconnaissance or data collection activity.</t>
+        </is>
+      </c>
+      <c r="L389" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M389" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N389" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O389" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>AN0455</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>discovery</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>T1201</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>Password Policy Discovery</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>DET0161</t>
+        </is>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>Password Policy Discovery via Command Line</t>
+        </is>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>host-local feeds only</t>
+        </is>
+      </c>
+      <c r="J390" t="inlineStr">
+        <is>
+          <t>WinEventLog:Security; WinEventLog:Sysmon</t>
+        </is>
+      </c>
+      <c r="K390" t="inlineStr">
+        <is>
+          <t>Detects adversarial query commands to discover system or domain password policy requirements (net accounts).</t>
+        </is>
+      </c>
+      <c r="L390" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M390" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N390" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O390" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refactored command-and-control rules to support multi-logsource splits and updated tracker
</commit_message>
<xml_diff>
--- a/ocsf_mapped_new_sprint.xlsx
+++ b/ocsf_mapped_new_sprint.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O390"/>
+  <dimension ref="A1:O399"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27858,6 +27858,663 @@
         </is>
       </c>
     </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>AN0100</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>command-and-control</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>T1102.002</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>Web Service: Bidirectional Communication</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>DET0035</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t>Bidirectional C2 Communication via Web Service API</t>
+        </is>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="J391" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 3, Event ID 4104</t>
+        </is>
+      </c>
+      <c r="K391" t="inlineStr">
+        <is>
+          <t>Detects command-line interpreters or scripting hosts initiating network connections to common web service API domains used for bidirectional C2 communication.</t>
+        </is>
+      </c>
+      <c r="L391" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M391" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N391" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O391" t="inlineStr"/>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>AN0109</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>command-and-control</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>T1568</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>Dynamic Resolution</t>
+        </is>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>DET0039</t>
+        </is>
+      </c>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>DNS Query from Non-Network System Utility</t>
+        </is>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="J392" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 3, Event ID 1</t>
+        </is>
+      </c>
+      <c r="K392" t="inlineStr">
+        <is>
+          <t>Detects network connections targeting DNS port 53 or suspicious process creation of non-network system utilities.</t>
+        </is>
+      </c>
+      <c r="L392" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M392" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N392" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O392" t="inlineStr"/>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>AN0158</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>command-and-control</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>T1102.001</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>Web Service: Dead Drop Resolver</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>DET0058</t>
+        </is>
+      </c>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t>Scripting Host Query to Dead Drop Web Service</t>
+        </is>
+      </c>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="J393" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 3, Event ID 4104</t>
+        </is>
+      </c>
+      <c r="K393" t="inlineStr">
+        <is>
+          <t>Detects scripting hosts or system processes initiating network connections or queries to known dead drop resolver domains.</t>
+        </is>
+      </c>
+      <c r="L393" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M393" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N393" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O393" t="inlineStr"/>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>AN0165</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>command-and-control</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>T1105</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>Ingress Tool Transfer</t>
+        </is>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>DET0060</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>Ingress Tool Transfer via CLI</t>
+        </is>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="J394" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1, Event ID 3, Event ID 4104</t>
+        </is>
+      </c>
+      <c r="K394" t="inlineStr">
+        <is>
+          <t>Detects command-line execution of tools performing ingress tool transfers from external locations.</t>
+        </is>
+      </c>
+      <c r="L394" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M394" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N394" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O394" t="inlineStr"/>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>AN0400</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>command-and-control</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>T1573.001</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>Encrypted Channel: Symmetric Cryptography</t>
+        </is>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>DET0143</t>
+        </is>
+      </c>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>Cryptographic DLL Loaded by Non-Cryptographic Process</t>
+        </is>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="J395" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 7, Event ID 3</t>
+        </is>
+      </c>
+      <c r="K395" t="inlineStr">
+        <is>
+          <t>Detects standard system applications loading Windows cryptographic DLLs or initiating network connections post-injection.</t>
+        </is>
+      </c>
+      <c r="L395" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M395" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N395" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O395" t="inlineStr"/>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>AN0633</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>command-and-control</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>T1571</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>Non-Standard Port</t>
+        </is>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>DET0227</t>
+        </is>
+      </c>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>Outbound Network Connection via Non-Standard Port</t>
+        </is>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="J396" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 3, Event ID 1</t>
+        </is>
+      </c>
+      <c r="K396" t="inlineStr">
+        <is>
+          <t>Detects outbound network connections initiated by system processes or office applications on atypical/non-standard port ranges.</t>
+        </is>
+      </c>
+      <c r="L396" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M396" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N396" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O396" t="inlineStr"/>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>AN0637</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>command-and-control</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>T1104</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>Multi-Stage Channels</t>
+        </is>
+      </c>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>DET0228</t>
+        </is>
+      </c>
+      <c r="H397" t="inlineStr">
+        <is>
+          <t>Multi-Stage C2 Channel Process spawning with Network Connection</t>
+        </is>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="J397" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 3, Event ID 1</t>
+        </is>
+      </c>
+      <c r="K397" t="inlineStr">
+        <is>
+          <t>Detects process creation patterns typical of multi-stage C2 channels, where a scripting host spawns an unexpected child process that immediately initiates outbound network connections.</t>
+        </is>
+      </c>
+      <c r="L397" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M397" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N397" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O397" t="inlineStr"/>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>AN0714</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>command-and-control</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>T1219</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>Remote Access Software</t>
+        </is>
+      </c>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>DET0259</t>
+        </is>
+      </c>
+      <c r="H398" t="inlineStr">
+        <is>
+          <t>Unauthorized Remote Management and Monitoring Software Execution</t>
+        </is>
+      </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="J398" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1, Event ID 3</t>
+        </is>
+      </c>
+      <c r="K398" t="inlineStr">
+        <is>
+          <t>Detects the execution of known Remote Management and Monitoring (RMM) or Remote Desktop software on unauthorized endpoints.</t>
+        </is>
+      </c>
+      <c r="L398" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M398" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N398" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O398" t="inlineStr"/>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>AN0728</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>command-and-control</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>T1568.003</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>Dynamic Resolution: DNS Calculation</t>
+        </is>
+      </c>
+      <c r="G399" t="inlineStr">
+        <is>
+          <t>DET0262</t>
+        </is>
+      </c>
+      <c r="H399" t="inlineStr">
+        <is>
+          <t>DNS TXT Query from Scripting Host</t>
+        </is>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="J399" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1, Event ID 4104</t>
+        </is>
+      </c>
+      <c r="K399" t="inlineStr">
+        <is>
+          <t>Detects DNS queries requesting TXT records initiated by scripting hosts or command line utilities.</t>
+        </is>
+      </c>
+      <c r="L399" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M399" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N399" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O399" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refactor Credential Access tactic rules to support split rules across multiple log sources
</commit_message>
<xml_diff>
--- a/ocsf_mapped_new_sprint.xlsx
+++ b/ocsf_mapped_new_sprint.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O399"/>
+  <dimension ref="A1:O409"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -576,7 +576,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -649,7 +648,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -722,7 +720,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -795,7 +792,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -868,7 +864,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -941,7 +936,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1014,7 +1008,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1087,7 +1080,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1160,7 +1152,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1233,7 +1224,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1306,7 +1296,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1379,7 +1368,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1452,7 +1440,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1525,7 +1512,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1598,7 +1584,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1671,7 +1656,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1744,7 +1728,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1817,7 +1800,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1890,7 +1872,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1963,7 +1944,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2036,7 +2016,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2109,7 +2088,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2182,7 +2160,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2255,7 +2232,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2328,7 +2304,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2396,8 +2371,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2465,8 +2438,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2534,8 +2505,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2603,8 +2572,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2672,8 +2639,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2741,8 +2706,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2810,8 +2773,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2879,8 +2840,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2948,8 +2907,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3017,8 +2974,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3086,8 +3041,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3160,7 +3113,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3228,8 +3180,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3297,8 +3247,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3366,8 +3314,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3435,8 +3381,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3504,8 +3448,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3573,8 +3515,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3642,8 +3582,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3711,8 +3649,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N46" t="inlineStr"/>
-      <c r="O46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3780,8 +3716,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N47" t="inlineStr"/>
-      <c r="O47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3849,8 +3783,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3918,8 +3850,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N49" t="inlineStr"/>
-      <c r="O49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3987,8 +3917,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -4056,8 +3984,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N51" t="inlineStr"/>
-      <c r="O51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4125,8 +4051,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4194,8 +4118,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N53" t="inlineStr"/>
-      <c r="O53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4263,8 +4185,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N54" t="inlineStr"/>
-      <c r="O54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4332,8 +4252,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N55" t="inlineStr"/>
-      <c r="O55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4401,8 +4319,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N56" t="inlineStr"/>
-      <c r="O56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4470,8 +4386,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N57" t="inlineStr"/>
-      <c r="O57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4539,8 +4453,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N58" t="inlineStr"/>
-      <c r="O58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -4608,8 +4520,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N59" t="inlineStr"/>
-      <c r="O59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4677,8 +4587,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N60" t="inlineStr"/>
-      <c r="O60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4746,8 +4654,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N61" t="inlineStr"/>
-      <c r="O61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4815,8 +4721,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N62" t="inlineStr"/>
-      <c r="O62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4884,8 +4788,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N63" t="inlineStr"/>
-      <c r="O63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4953,8 +4855,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N64" t="inlineStr"/>
-      <c r="O64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5022,8 +4922,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N65" t="inlineStr"/>
-      <c r="O65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5091,8 +4989,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N66" t="inlineStr"/>
-      <c r="O66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5160,8 +5056,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N67" t="inlineStr"/>
-      <c r="O67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -5229,8 +5123,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N68" t="inlineStr"/>
-      <c r="O68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5298,8 +5190,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N69" t="inlineStr"/>
-      <c r="O69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5367,8 +5257,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N70" t="inlineStr"/>
-      <c r="O70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5436,8 +5324,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N71" t="inlineStr"/>
-      <c r="O71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -5505,8 +5391,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N72" t="inlineStr"/>
-      <c r="O72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -5574,8 +5458,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N73" t="inlineStr"/>
-      <c r="O73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -5643,8 +5525,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N74" t="inlineStr"/>
-      <c r="O74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -5712,8 +5592,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N75" t="inlineStr"/>
-      <c r="O75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -5781,8 +5659,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N76" t="inlineStr"/>
-      <c r="O76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -5850,8 +5726,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N77" t="inlineStr"/>
-      <c r="O77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -5919,8 +5793,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N78" t="inlineStr"/>
-      <c r="O78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -5988,8 +5860,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N79" t="inlineStr"/>
-      <c r="O79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -6057,8 +5927,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N80" t="inlineStr"/>
-      <c r="O80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -6126,8 +5994,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N81" t="inlineStr"/>
-      <c r="O81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -6195,8 +6061,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N82" t="inlineStr"/>
-      <c r="O82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -6264,8 +6128,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N83" t="inlineStr"/>
-      <c r="O83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -6333,8 +6195,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N84" t="inlineStr"/>
-      <c r="O84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -6402,8 +6262,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N85" t="inlineStr"/>
-      <c r="O85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -6471,8 +6329,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N86" t="inlineStr"/>
-      <c r="O86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -6540,8 +6396,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N87" t="inlineStr"/>
-      <c r="O87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -6609,8 +6463,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N88" t="inlineStr"/>
-      <c r="O88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -6678,8 +6530,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N89" t="inlineStr"/>
-      <c r="O89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -6747,8 +6597,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N90" t="inlineStr"/>
-      <c r="O90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -6816,8 +6664,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N91" t="inlineStr"/>
-      <c r="O91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -6885,8 +6731,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N92" t="inlineStr"/>
-      <c r="O92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -6954,8 +6798,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N93" t="inlineStr"/>
-      <c r="O93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -7023,8 +6865,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N94" t="inlineStr"/>
-      <c r="O94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -7092,8 +6932,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N95" t="inlineStr"/>
-      <c r="O95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -7161,8 +6999,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N96" t="inlineStr"/>
-      <c r="O96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -7230,8 +7066,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N97" t="inlineStr"/>
-      <c r="O97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -7299,8 +7133,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N98" t="inlineStr"/>
-      <c r="O98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -7368,8 +7200,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N99" t="inlineStr"/>
-      <c r="O99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -7437,8 +7267,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N100" t="inlineStr"/>
-      <c r="O100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -7506,8 +7334,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N101" t="inlineStr"/>
-      <c r="O101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -7575,8 +7401,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N102" t="inlineStr"/>
-      <c r="O102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -7644,8 +7468,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N103" t="inlineStr"/>
-      <c r="O103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -7713,8 +7535,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N104" t="inlineStr"/>
-      <c r="O104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -7782,8 +7602,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N105" t="inlineStr"/>
-      <c r="O105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -7851,8 +7669,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N106" t="inlineStr"/>
-      <c r="O106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -7920,8 +7736,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N107" t="inlineStr"/>
-      <c r="O107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -7989,8 +7803,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N108" t="inlineStr"/>
-      <c r="O108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -8058,8 +7870,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N109" t="inlineStr"/>
-      <c r="O109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -8127,8 +7937,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N110" t="inlineStr"/>
-      <c r="O110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -8201,7 +8009,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -8274,7 +8081,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -8347,7 +8153,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -8420,7 +8225,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -8493,7 +8297,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -8566,7 +8369,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -8639,7 +8441,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -8712,7 +8513,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -8785,7 +8585,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -8858,7 +8657,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -8931,7 +8729,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -9004,7 +8801,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -9077,7 +8873,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -9150,7 +8945,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -9223,7 +9017,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -9296,7 +9089,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -9369,7 +9161,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -9442,7 +9233,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -9510,8 +9300,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N129" t="inlineStr"/>
-      <c r="O129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -9579,8 +9367,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N130" t="inlineStr"/>
-      <c r="O130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -9648,8 +9434,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N131" t="inlineStr"/>
-      <c r="O131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -9717,8 +9501,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N132" t="inlineStr"/>
-      <c r="O132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -9786,8 +9568,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N133" t="inlineStr"/>
-      <c r="O133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -9855,8 +9635,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N134" t="inlineStr"/>
-      <c r="O134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -9924,8 +9702,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N135" t="inlineStr"/>
-      <c r="O135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -9993,8 +9769,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N136" t="inlineStr"/>
-      <c r="O136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -10062,8 +9836,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N137" t="inlineStr"/>
-      <c r="O137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -10131,8 +9903,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N138" t="inlineStr"/>
-      <c r="O138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -10200,8 +9970,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N139" t="inlineStr"/>
-      <c r="O139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -10269,8 +10037,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N140" t="inlineStr"/>
-      <c r="O140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -10338,8 +10104,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N141" t="inlineStr"/>
-      <c r="O141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -10407,8 +10171,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N142" t="inlineStr"/>
-      <c r="O142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -10476,8 +10238,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N143" t="inlineStr"/>
-      <c r="O143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -10545,8 +10305,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N144" t="inlineStr"/>
-      <c r="O144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -10614,8 +10372,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N145" t="inlineStr"/>
-      <c r="O145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -10683,8 +10439,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N146" t="inlineStr"/>
-      <c r="O146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -10752,8 +10506,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N147" t="inlineStr"/>
-      <c r="O147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -10821,8 +10573,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N148" t="inlineStr"/>
-      <c r="O148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -10890,8 +10640,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N149" t="inlineStr"/>
-      <c r="O149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -10959,8 +10707,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N150" t="inlineStr"/>
-      <c r="O150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -11028,8 +10774,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N151" t="inlineStr"/>
-      <c r="O151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -11097,8 +10841,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N152" t="inlineStr"/>
-      <c r="O152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -11166,8 +10908,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N153" t="inlineStr"/>
-      <c r="O153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -11235,8 +10975,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N154" t="inlineStr"/>
-      <c r="O154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -11304,8 +11042,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N155" t="inlineStr"/>
-      <c r="O155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -11373,8 +11109,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N156" t="inlineStr"/>
-      <c r="O156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -11442,8 +11176,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N157" t="inlineStr"/>
-      <c r="O157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -11511,8 +11243,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N158" t="inlineStr"/>
-      <c r="O158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -11580,8 +11310,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N159" t="inlineStr"/>
-      <c r="O159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -11649,8 +11377,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N160" t="inlineStr"/>
-      <c r="O160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -11718,8 +11444,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N161" t="inlineStr"/>
-      <c r="O161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -11787,8 +11511,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N162" t="inlineStr"/>
-      <c r="O162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -11856,8 +11578,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N163" t="inlineStr"/>
-      <c r="O163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -11925,8 +11645,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N164" t="inlineStr"/>
-      <c r="O164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -11994,8 +11712,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N165" t="inlineStr"/>
-      <c r="O165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -12063,8 +11779,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N166" t="inlineStr"/>
-      <c r="O166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -12132,8 +11846,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N167" t="inlineStr"/>
-      <c r="O167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -12201,8 +11913,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N168" t="inlineStr"/>
-      <c r="O168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -12270,8 +11980,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N169" t="inlineStr"/>
-      <c r="O169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -12339,8 +12047,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N170" t="inlineStr"/>
-      <c r="O170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -12408,8 +12114,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N171" t="inlineStr"/>
-      <c r="O171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -12477,8 +12181,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N172" t="inlineStr"/>
-      <c r="O172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -12546,8 +12248,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N173" t="inlineStr"/>
-      <c r="O173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -12615,8 +12315,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N174" t="inlineStr"/>
-      <c r="O174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -12684,8 +12382,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N175" t="inlineStr"/>
-      <c r="O175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -12753,8 +12449,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N176" t="inlineStr"/>
-      <c r="O176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -12822,8 +12516,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N177" t="inlineStr"/>
-      <c r="O177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -12891,8 +12583,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N178" t="inlineStr"/>
-      <c r="O178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -12960,8 +12650,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N179" t="inlineStr"/>
-      <c r="O179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -13029,8 +12717,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N180" t="inlineStr"/>
-      <c r="O180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -13098,8 +12784,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N181" t="inlineStr"/>
-      <c r="O181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -13167,8 +12851,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N182" t="inlineStr"/>
-      <c r="O182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -13236,8 +12918,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N183" t="inlineStr"/>
-      <c r="O183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -13305,8 +12985,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N184" t="inlineStr"/>
-      <c r="O184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -13374,8 +13052,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N185" t="inlineStr"/>
-      <c r="O185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -13443,8 +13119,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N186" t="inlineStr"/>
-      <c r="O186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -13512,8 +13186,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N187" t="inlineStr"/>
-      <c r="O187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -13581,8 +13253,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N188" t="inlineStr"/>
-      <c r="O188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -13650,8 +13320,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N189" t="inlineStr"/>
-      <c r="O189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -13719,8 +13387,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N190" t="inlineStr"/>
-      <c r="O190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -13788,8 +13454,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N191" t="inlineStr"/>
-      <c r="O191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -13857,8 +13521,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N192" t="inlineStr"/>
-      <c r="O192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -13926,8 +13588,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N193" t="inlineStr"/>
-      <c r="O193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -13995,8 +13655,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N194" t="inlineStr"/>
-      <c r="O194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -14064,8 +13722,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N195" t="inlineStr"/>
-      <c r="O195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -14133,8 +13789,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N196" t="inlineStr"/>
-      <c r="O196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -14202,8 +13856,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N197" t="inlineStr"/>
-      <c r="O197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -14271,8 +13923,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N198" t="inlineStr"/>
-      <c r="O198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -14340,8 +13990,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N199" t="inlineStr"/>
-      <c r="O199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -14409,8 +14057,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N200" t="inlineStr"/>
-      <c r="O200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -14478,8 +14124,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N201" t="inlineStr"/>
-      <c r="O201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -14547,8 +14191,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N202" t="inlineStr"/>
-      <c r="O202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -14616,8 +14258,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N203" t="inlineStr"/>
-      <c r="O203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -14685,8 +14325,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N204" t="inlineStr"/>
-      <c r="O204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -14754,8 +14392,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N205" t="inlineStr"/>
-      <c r="O205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -14823,8 +14459,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N206" t="inlineStr"/>
-      <c r="O206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -14892,8 +14526,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N207" t="inlineStr"/>
-      <c r="O207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -14961,8 +14593,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N208" t="inlineStr"/>
-      <c r="O208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -15030,8 +14660,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N209" t="inlineStr"/>
-      <c r="O209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -15099,8 +14727,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N210" t="inlineStr"/>
-      <c r="O210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -15168,8 +14794,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N211" t="inlineStr"/>
-      <c r="O211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -15237,8 +14861,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N212" t="inlineStr"/>
-      <c r="O212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -15306,8 +14928,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N213" t="inlineStr"/>
-      <c r="O213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -15375,8 +14995,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N214" t="inlineStr"/>
-      <c r="O214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -15444,8 +15062,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N215" t="inlineStr"/>
-      <c r="O215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -15513,8 +15129,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N216" t="inlineStr"/>
-      <c r="O216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -15582,8 +15196,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N217" t="inlineStr"/>
-      <c r="O217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -15651,8 +15263,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N218" t="inlineStr"/>
-      <c r="O218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -15720,8 +15330,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N219" t="inlineStr"/>
-      <c r="O219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -15789,8 +15397,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N220" t="inlineStr"/>
-      <c r="O220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -16166,8 +15772,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N225" t="inlineStr"/>
-      <c r="O225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -16235,8 +15839,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N226" t="inlineStr"/>
-      <c r="O226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -16304,8 +15906,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N227" t="inlineStr"/>
-      <c r="O227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -16373,8 +15973,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N228" t="inlineStr"/>
-      <c r="O228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -16442,8 +16040,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N229" t="inlineStr"/>
-      <c r="O229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -16511,8 +16107,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N230" t="inlineStr"/>
-      <c r="O230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -16580,8 +16174,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N231" t="inlineStr"/>
-      <c r="O231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -16649,8 +16241,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N232" t="inlineStr"/>
-      <c r="O232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -16718,8 +16308,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N233" t="inlineStr"/>
-      <c r="O233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -16787,8 +16375,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N234" t="inlineStr"/>
-      <c r="O234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -16856,8 +16442,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N235" t="inlineStr"/>
-      <c r="O235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -16925,8 +16509,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N236" t="inlineStr"/>
-      <c r="O236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -16994,8 +16576,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N237" t="inlineStr"/>
-      <c r="O237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -17063,8 +16643,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N238" t="inlineStr"/>
-      <c r="O238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -17132,8 +16710,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N239" t="inlineStr"/>
-      <c r="O239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -17201,8 +16777,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N240" t="inlineStr"/>
-      <c r="O240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -17270,8 +16844,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N241" t="inlineStr"/>
-      <c r="O241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -17339,8 +16911,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N242" t="inlineStr"/>
-      <c r="O242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -17408,8 +16978,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N243" t="inlineStr"/>
-      <c r="O243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -17477,8 +17045,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N244" t="inlineStr"/>
-      <c r="O244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -17546,8 +17112,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N245" t="inlineStr"/>
-      <c r="O245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -17615,8 +17179,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N246" t="inlineStr"/>
-      <c r="O246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -17684,8 +17246,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N247" t="inlineStr"/>
-      <c r="O247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -17753,8 +17313,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N248" t="inlineStr"/>
-      <c r="O248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -17822,8 +17380,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N249" t="inlineStr"/>
-      <c r="O249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -17891,8 +17447,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N250" t="inlineStr"/>
-      <c r="O250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -17960,8 +17514,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N251" t="inlineStr"/>
-      <c r="O251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -18029,8 +17581,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N252" t="inlineStr"/>
-      <c r="O252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -18098,8 +17648,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N253" t="inlineStr"/>
-      <c r="O253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -18167,8 +17715,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N254" t="inlineStr"/>
-      <c r="O254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -18236,8 +17782,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N255" t="inlineStr"/>
-      <c r="O255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -18305,8 +17849,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N256" t="inlineStr"/>
-      <c r="O256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -18374,8 +17916,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N257" t="inlineStr"/>
-      <c r="O257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -18443,8 +17983,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N258" t="inlineStr"/>
-      <c r="O258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -18512,8 +18050,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N259" t="inlineStr"/>
-      <c r="O259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -18581,8 +18117,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N260" t="inlineStr"/>
-      <c r="O260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -18650,8 +18184,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N261" t="inlineStr"/>
-      <c r="O261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -18719,8 +18251,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N262" t="inlineStr"/>
-      <c r="O262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -18788,8 +18318,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N263" t="inlineStr"/>
-      <c r="O263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -18857,8 +18385,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N264" t="inlineStr"/>
-      <c r="O264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -18926,8 +18452,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N265" t="inlineStr"/>
-      <c r="O265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -18995,8 +18519,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N266" t="inlineStr"/>
-      <c r="O266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -19064,8 +18586,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N267" t="inlineStr"/>
-      <c r="O267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -19133,8 +18653,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N268" t="inlineStr"/>
-      <c r="O268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -19202,8 +18720,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N269" t="inlineStr"/>
-      <c r="O269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -19271,8 +18787,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N270" t="inlineStr"/>
-      <c r="O270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -19340,8 +18854,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N271" t="inlineStr"/>
-      <c r="O271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -19409,8 +18921,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N272" t="inlineStr"/>
-      <c r="O272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -19478,8 +18988,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N273" t="inlineStr"/>
-      <c r="O273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -19547,8 +19055,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N274" t="inlineStr"/>
-      <c r="O274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -19616,8 +19122,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N275" t="inlineStr"/>
-      <c r="O275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -19685,8 +19189,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N276" t="inlineStr"/>
-      <c r="O276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -19754,8 +19256,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N277" t="inlineStr"/>
-      <c r="O277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -19823,8 +19323,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N278" t="inlineStr"/>
-      <c r="O278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -19974,7 +19472,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -20047,7 +19544,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O281" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -20120,7 +19616,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -20193,7 +19688,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -20266,7 +19760,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O284" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -20339,7 +19832,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O285" t="inlineStr"/>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -20412,7 +19904,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O286" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -20485,7 +19976,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O287" t="inlineStr"/>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -20558,7 +20048,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O288" t="inlineStr"/>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -20631,7 +20120,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O289" t="inlineStr"/>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -20704,7 +20192,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O290" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -20777,7 +20264,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O291" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -20850,7 +20336,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O292" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -20923,7 +20408,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O293" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -20996,7 +20480,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O294" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -21069,7 +20552,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -21142,7 +20624,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O296" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -21215,7 +20696,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O297" t="inlineStr"/>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -21288,7 +20768,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O298" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -21361,7 +20840,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O299" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -21434,7 +20912,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O300" t="inlineStr"/>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -21507,7 +20984,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O301" t="inlineStr"/>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -21580,7 +21056,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O302" t="inlineStr"/>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -21653,7 +21128,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O303" t="inlineStr"/>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -21726,7 +21200,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O304" t="inlineStr"/>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -21799,7 +21272,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O305" t="inlineStr"/>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -21867,8 +21339,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N306" t="inlineStr"/>
-      <c r="O306" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -21936,8 +21406,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N307" t="inlineStr"/>
-      <c r="O307" t="inlineStr"/>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -22005,8 +21473,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N308" t="inlineStr"/>
-      <c r="O308" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -22074,8 +21540,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N309" t="inlineStr"/>
-      <c r="O309" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -22143,8 +21607,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N310" t="inlineStr"/>
-      <c r="O310" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -22212,8 +21674,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N311" t="inlineStr"/>
-      <c r="O311" t="inlineStr"/>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -22281,8 +21741,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N312" t="inlineStr"/>
-      <c r="O312" t="inlineStr"/>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -22350,8 +21808,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N313" t="inlineStr"/>
-      <c r="O313" t="inlineStr"/>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -22419,8 +21875,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N314" t="inlineStr"/>
-      <c r="O314" t="inlineStr"/>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -22488,8 +21942,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N315" t="inlineStr"/>
-      <c r="O315" t="inlineStr"/>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -22557,8 +22009,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N316" t="inlineStr"/>
-      <c r="O316" t="inlineStr"/>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -22626,8 +22076,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N317" t="inlineStr"/>
-      <c r="O317" t="inlineStr"/>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -22695,8 +22143,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N318" t="inlineStr"/>
-      <c r="O318" t="inlineStr"/>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -22764,8 +22210,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N319" t="inlineStr"/>
-      <c r="O319" t="inlineStr"/>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -22833,8 +22277,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N320" t="inlineStr"/>
-      <c r="O320" t="inlineStr"/>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -22902,8 +22344,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N321" t="inlineStr"/>
-      <c r="O321" t="inlineStr"/>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -22971,8 +22411,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N322" t="inlineStr"/>
-      <c r="O322" t="inlineStr"/>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -23040,8 +22478,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N323" t="inlineStr"/>
-      <c r="O323" t="inlineStr"/>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -23109,8 +22545,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N324" t="inlineStr"/>
-      <c r="O324" t="inlineStr"/>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -23178,8 +22612,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N325" t="inlineStr"/>
-      <c r="O325" t="inlineStr"/>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -23247,8 +22679,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N326" t="inlineStr"/>
-      <c r="O326" t="inlineStr"/>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -23316,8 +22746,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N327" t="inlineStr"/>
-      <c r="O327" t="inlineStr"/>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -23385,8 +22813,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N328" t="inlineStr"/>
-      <c r="O328" t="inlineStr"/>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -23454,8 +22880,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N329" t="inlineStr"/>
-      <c r="O329" t="inlineStr"/>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -23523,8 +22947,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N330" t="inlineStr"/>
-      <c r="O330" t="inlineStr"/>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -23592,8 +23014,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N331" t="inlineStr"/>
-      <c r="O331" t="inlineStr"/>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -23661,8 +23081,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N332" t="inlineStr"/>
-      <c r="O332" t="inlineStr"/>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -23730,8 +23148,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N333" t="inlineStr"/>
-      <c r="O333" t="inlineStr"/>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -23799,8 +23215,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N334" t="inlineStr"/>
-      <c r="O334" t="inlineStr"/>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -23868,8 +23282,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N335" t="inlineStr"/>
-      <c r="O335" t="inlineStr"/>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -23937,8 +23349,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N336" t="inlineStr"/>
-      <c r="O336" t="inlineStr"/>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -24011,7 +23421,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O337" t="inlineStr"/>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -24084,7 +23493,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O338" t="inlineStr"/>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -24157,7 +23565,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O339" t="inlineStr"/>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -24230,7 +23637,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O340" t="inlineStr"/>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -24303,7 +23709,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O341" t="inlineStr"/>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -24376,7 +23781,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O342" t="inlineStr"/>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -24449,7 +23853,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O343" t="inlineStr"/>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -24517,8 +23920,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N344" t="inlineStr"/>
-      <c r="O344" t="inlineStr"/>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -24586,8 +23987,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N345" t="inlineStr"/>
-      <c r="O345" t="inlineStr"/>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -24655,8 +24054,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N346" t="inlineStr"/>
-      <c r="O346" t="inlineStr"/>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -24724,8 +24121,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N347" t="inlineStr"/>
-      <c r="O347" t="inlineStr"/>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -24793,8 +24188,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N348" t="inlineStr"/>
-      <c r="O348" t="inlineStr"/>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -24862,8 +24255,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N349" t="inlineStr"/>
-      <c r="O349" t="inlineStr"/>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -24931,8 +24322,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N350" t="inlineStr"/>
-      <c r="O350" t="inlineStr"/>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -25000,8 +24389,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N351" t="inlineStr"/>
-      <c r="O351" t="inlineStr"/>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -25069,8 +24456,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N352" t="inlineStr"/>
-      <c r="O352" t="inlineStr"/>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
@@ -25138,8 +24523,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N353" t="inlineStr"/>
-      <c r="O353" t="inlineStr"/>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -25207,8 +24590,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N354" t="inlineStr"/>
-      <c r="O354" t="inlineStr"/>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -25276,8 +24657,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N355" t="inlineStr"/>
-      <c r="O355" t="inlineStr"/>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -25345,8 +24724,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N356" t="inlineStr"/>
-      <c r="O356" t="inlineStr"/>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -25414,8 +24791,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N357" t="inlineStr"/>
-      <c r="O357" t="inlineStr"/>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -25483,8 +24858,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N358" t="inlineStr"/>
-      <c r="O358" t="inlineStr"/>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -25552,8 +24925,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N359" t="inlineStr"/>
-      <c r="O359" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -25621,8 +24992,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N360" t="inlineStr"/>
-      <c r="O360" t="inlineStr"/>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -25690,8 +25059,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N361" t="inlineStr"/>
-      <c r="O361" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -25759,8 +25126,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N362" t="inlineStr"/>
-      <c r="O362" t="inlineStr"/>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -25828,8 +25193,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N363" t="inlineStr"/>
-      <c r="O363" t="inlineStr"/>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -25902,7 +25265,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O364" t="inlineStr"/>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -25975,7 +25337,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O365" t="inlineStr"/>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -26048,7 +25409,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O366" t="inlineStr"/>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -26121,7 +25481,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O367" t="inlineStr"/>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -26194,7 +25553,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O368" t="inlineStr"/>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -26267,7 +25625,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O369" t="inlineStr"/>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
@@ -26340,7 +25697,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O370" t="inlineStr"/>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
@@ -26413,7 +25769,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O371" t="inlineStr"/>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
@@ -26486,7 +25841,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O372" t="inlineStr"/>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
@@ -26559,7 +25913,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O373" t="inlineStr"/>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
@@ -26632,7 +25985,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O374" t="inlineStr"/>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
@@ -26705,7 +26057,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O375" t="inlineStr"/>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
@@ -26778,7 +26129,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O376" t="inlineStr"/>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
@@ -27929,7 +27279,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O391" t="inlineStr"/>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
@@ -28002,7 +27351,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O392" t="inlineStr"/>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
@@ -28075,7 +27423,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O393" t="inlineStr"/>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
@@ -28148,7 +27495,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O394" t="inlineStr"/>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
@@ -28221,7 +27567,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O395" t="inlineStr"/>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
@@ -28294,7 +27639,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O396" t="inlineStr"/>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
@@ -28367,7 +27711,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O397" t="inlineStr"/>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
@@ -28440,7 +27783,6 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O398" t="inlineStr"/>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
@@ -28513,7 +27855,726 @@
           <t>done</t>
         </is>
       </c>
-      <c r="O399" t="inlineStr"/>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>AN0105</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>credential-access</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>T1555.003</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>Credentials from Password Stores: Credentials from Web Browsers</t>
+        </is>
+      </c>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>DET0037</t>
+        </is>
+      </c>
+      <c r="H400" t="inlineStr">
+        <is>
+          <t>Suspicious Browser Credential Store Access</t>
+        </is>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="J400" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1, Event ID 11</t>
+        </is>
+      </c>
+      <c r="K400" t="inlineStr">
+        <is>
+          <t>Detects command-line operations or file events attempting to copy, compress, or access web browser credential and cookie databases, indicating potential credential theft.</t>
+        </is>
+      </c>
+      <c r="L400" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M400" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N400" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>AN0235</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>credential-access</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>T1003.002</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>OS Credential Dumping: Security Account Manager</t>
+        </is>
+      </c>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>DET0085</t>
+        </is>
+      </c>
+      <c r="H401" t="inlineStr">
+        <is>
+          <t>Suspicious SAM Registry Hive Export</t>
+        </is>
+      </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="J401" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1, Event ID 13, Event ID 11</t>
+        </is>
+      </c>
+      <c r="K401" t="inlineStr">
+        <is>
+          <t>Detects attempts to save/export the SAM registry hive via command line, registry events, or raw file copies.</t>
+        </is>
+      </c>
+      <c r="L401" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M401" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N401" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>AN0287</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>credential-access</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>T1556</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>Modify Authentication Process</t>
+        </is>
+      </c>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>DET0104</t>
+        </is>
+      </c>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>Suspicious LSA Authentication Package Modification</t>
+        </is>
+      </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="J402" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 13, Event ID 1</t>
+        </is>
+      </c>
+      <c r="K402" t="inlineStr">
+        <is>
+          <t>Detects registry set modifications or command line operations adding new LSA packages or notification filters.</t>
+        </is>
+      </c>
+      <c r="L402" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M402" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N402" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>AN0292</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>credential-access</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>T1110.002</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>Brute Force: Password Cracking</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>DET0105</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>Local Password Cracking Activity</t>
+        </is>
+      </c>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="J403" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1, Event ID 4104</t>
+        </is>
+      </c>
+      <c r="K403" t="inlineStr">
+        <is>
+          <t>Detects the execution of known password cracking utilities or command-line arguments on a local endpoint.</t>
+        </is>
+      </c>
+      <c r="L403" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M403" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N403" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>AN0316</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>credential-access</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>T1558.004</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>Steal or Forge Kerberos Tickets: AS-REP Roasting</t>
+        </is>
+      </c>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>DET0113</t>
+        </is>
+      </c>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t>AS-REP Roasting Tool Execution</t>
+        </is>
+      </c>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="J404" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1, Event ID 4104</t>
+        </is>
+      </c>
+      <c r="K404" t="inlineStr">
+        <is>
+          <t>Detects command-line parameters and script blocks associated with AS-REP Roasting attacks.</t>
+        </is>
+      </c>
+      <c r="L404" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M404" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N404" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>AN0378</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>credential-access</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>T1555.004</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>Credentials from Password Stores: Windows Credential Manager</t>
+        </is>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>DET0134</t>
+        </is>
+      </c>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t>Suspicious Windows Credential Manager Access</t>
+        </is>
+      </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="J405" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1, Event ID 4104</t>
+        </is>
+      </c>
+      <c r="K405" t="inlineStr">
+        <is>
+          <t>Detects command-line operations or scripting blocks querying the Windows Credential Manager (Vault).</t>
+        </is>
+      </c>
+      <c r="L405" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M405" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N405" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>AN0405</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>credential-access</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>T1558.001</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>Steal or Forge Kerberos Tickets: Golden Ticket</t>
+        </is>
+      </c>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>DET0144</t>
+        </is>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>Golden Ticket Forging Tool Execution</t>
+        </is>
+      </c>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="J406" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1, Event ID 4104</t>
+        </is>
+      </c>
+      <c r="K406" t="inlineStr">
+        <is>
+          <t>Detects command-line parameters and process executions associated with the forging or injection of Kerberos Golden Tickets.</t>
+        </is>
+      </c>
+      <c r="L406" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M406" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N406" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>AN0420</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>credential-access</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>T1606.002</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>Forge Web Credentials: SAML Tokens</t>
+        </is>
+      </c>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>DET0148</t>
+        </is>
+      </c>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t>Suspicious AD FS Database Query for SAML Certificate Extraction</t>
+        </is>
+      </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="J407" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1, Event ID 4104</t>
+        </is>
+      </c>
+      <c r="K407" t="inlineStr">
+        <is>
+          <t>Detects command-line execution or script queries attempting to extract SAML signing certificates from WID.</t>
+        </is>
+      </c>
+      <c r="L407" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M407" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N407" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>AN0444</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>credential-access</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>T1558.003</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>Steal or Forge Kerberos Tickets: Kerberoasting</t>
+        </is>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>DET0157</t>
+        </is>
+      </c>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t>Suspicious SPN Enumeration and Kerberoasting Activity</t>
+        </is>
+      </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="J408" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1, Event ID 4104</t>
+        </is>
+      </c>
+      <c r="K408" t="inlineStr">
+        <is>
+          <t>Detects command-line parameters or script blocks associated with SPN enumeration and Kerberoasting.</t>
+        </is>
+      </c>
+      <c r="L408" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M408" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N408" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>AN0451</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>credential-access</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>T1621</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>Multi-Factor Authentication Request Generation</t>
+        </is>
+      </c>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t>DET0160</t>
+        </is>
+      </c>
+      <c r="H409" t="inlineStr">
+        <is>
+          <t>MFA Request Fatigue Generation</t>
+        </is>
+      </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="J409" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K409" t="inlineStr">
+        <is>
+          <t>This technique is not detectable from Sysmon, Windows Security, or Defender logs.</t>
+        </is>
+      </c>
+      <c r="L409" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M409" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N409" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Refactor Impact tactic rules to support split rules across multiple log sources
</commit_message>
<xml_diff>
--- a/ocsf_mapped_new_sprint.xlsx
+++ b/ocsf_mapped_new_sprint.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O409"/>
+  <dimension ref="A1:O419"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28576,6 +28576,726 @@
         </is>
       </c>
     </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>AN0061</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>impact</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>T1489</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>Service Stop</t>
+        </is>
+      </c>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>DET0021</t>
+        </is>
+      </c>
+      <c r="H410" t="inlineStr">
+        <is>
+          <t>Stopping or Disabling Critical System Services via CLI</t>
+        </is>
+      </c>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="J410" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1, Event ID 4104</t>
+        </is>
+      </c>
+      <c r="K410" t="inlineStr">
+        <is>
+          <t>Detects command-line execution of sc.exe, net.exe, or PowerShell cmdlets stopping or disabling critical system services (e.g. anti-virus, firewalls, databases).</t>
+        </is>
+      </c>
+      <c r="L410" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M410" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N410" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>AN0080</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>impact</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>T1496.002</t>
+        </is>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t>Resource Hijacking: Joint Resources</t>
+        </is>
+      </c>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>DET0028</t>
+        </is>
+      </c>
+      <c r="H411" t="inlineStr">
+        <is>
+          <t>Execution of Bandwidth Hijacking or Proxyjacking Software</t>
+        </is>
+      </c>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="J411" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1, Event ID 3</t>
+        </is>
+      </c>
+      <c r="K411" t="inlineStr">
+        <is>
+          <t>Detects command-line execution of known proxyjacking, bandwidth sharing, or botnet scanning software, which is used for bandwidth hijacking and resource abuse.</t>
+        </is>
+      </c>
+      <c r="L411" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M411" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N411" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>AN0162</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>impact</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>T1565</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>Data Manipulation</t>
+        </is>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>DET0162</t>
+        </is>
+      </c>
+      <c r="H412" t="inlineStr">
+        <is>
+          <t>Database or Log File Modification by Non-Database Process</t>
+        </is>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="J412" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 11, Event ID 1</t>
+        </is>
+      </c>
+      <c r="K412" t="inlineStr">
+        <is>
+          <t>Detects command-line interpreters or scripting hosts modifying or creating database files (e.g., .db, .sqlite, .mdf) or system log files (.evtx), which can indicate unauthorized data manipulation or log tempering.</t>
+        </is>
+      </c>
+      <c r="L412" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M412" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N412" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>AN0229</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>impact</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>T1491.001</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>Defacement: Internal Defacement</t>
+        </is>
+      </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>DET0082</t>
+        </is>
+      </c>
+      <c r="H413" t="inlineStr">
+        <is>
+          <t>Registry Modification for System Defacement</t>
+        </is>
+      </c>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="J413" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 13, Event ID 1</t>
+        </is>
+      </c>
+      <c r="K413" t="inlineStr">
+        <is>
+          <t>Detects command-line registry modifications targeting Windows logon legal notice banners or wallpaper registry values, which can indicate system defacement.</t>
+        </is>
+      </c>
+      <c r="L413" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M413" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N413" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>AN0334</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>impact</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>T1531</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>Account Access Removal</t>
+        </is>
+      </c>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t>DET0334</t>
+        </is>
+      </c>
+      <c r="H414" t="inlineStr">
+        <is>
+          <t>User Account Access Removal via CLI</t>
+        </is>
+      </c>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="J414" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1, Event ID 4104</t>
+        </is>
+      </c>
+      <c r="K414" t="inlineStr">
+        <is>
+          <t>Detects command-line execution of net.exe or PowerShell cmdlets used to delete, disable, or deactivate user accounts, which can be abused to lock out administrators.</t>
+        </is>
+      </c>
+      <c r="L414" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M414" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N414" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>AN0384</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>impact</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>T1561</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>Disk Wipe</t>
+        </is>
+      </c>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t>DET0384</t>
+        </is>
+      </c>
+      <c r="H415" t="inlineStr">
+        <is>
+          <t>Disk Wiping and Partition Destruction Utilities</t>
+        </is>
+      </c>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="J415" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1, Event ID 4104</t>
+        </is>
+      </c>
+      <c r="K415" t="inlineStr">
+        <is>
+          <t>Detects command-line execution of disk formatting, partition management, or raw volume dismounting tools (such as diskpart, format, fsutil) used in disk wiping.</t>
+        </is>
+      </c>
+      <c r="L415" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M415" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N415" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>AN0411</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>impact</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>T1485</t>
+        </is>
+      </c>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t>Data Destruction</t>
+        </is>
+      </c>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t>DET0146</t>
+        </is>
+      </c>
+      <c r="H416" t="inlineStr">
+        <is>
+          <t>File Wiping or Volume Shadow Copy Deletion</t>
+        </is>
+      </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="J416" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1, Event ID 4104</t>
+        </is>
+      </c>
+      <c r="K416" t="inlineStr">
+        <is>
+          <t>Detects command-line execution of tools used for data destruction, such as sdelete, cipher /w, or commands deleting Volume Shadow Copies (vssadmin, wmic).</t>
+        </is>
+      </c>
+      <c r="L416" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M416" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N416" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>AN0474</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>impact</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>T1495</t>
+        </is>
+      </c>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>Disable Status Recovery</t>
+        </is>
+      </c>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t>DET0167</t>
+        </is>
+      </c>
+      <c r="H417" t="inlineStr">
+        <is>
+          <t>Boot Configuration Tampering via Bcdedit</t>
+        </is>
+      </c>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="J417" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1, Event ID 4104</t>
+        </is>
+      </c>
+      <c r="K417" t="inlineStr">
+        <is>
+          <t>Detects command-line modifications using bcdedit.exe to disable boot recovery options, disable safe boot configurations, or set anomalous boot configurations, which is typical of destructive ransomware and system disruption.</t>
+        </is>
+      </c>
+      <c r="L417" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M417" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N417" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>AN0489</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>impact</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>T1499.002</t>
+        </is>
+      </c>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t>Endpoint Denial of Service: Service Exhaustion</t>
+        </is>
+      </c>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t>DET0173</t>
+        </is>
+      </c>
+      <c r="H418" t="inlineStr">
+        <is>
+          <t>Potential Endpoint Service Exhaustion Flood Tool Execution</t>
+        </is>
+      </c>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="J418" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1, Event ID 3</t>
+        </is>
+      </c>
+      <c r="K418" t="inlineStr">
+        <is>
+          <t>Detects the execution of known load testing or HTTP flooding utilities (like ab.exe or slowhttptest) or scripting engines running parameters indicative of a service exhaustion flood.</t>
+        </is>
+      </c>
+      <c r="L418" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M418" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N418" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>AN0555</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>impact</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>T1565.001</t>
+        </is>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>Data Manipulation: Stored Data Manipulation</t>
+        </is>
+      </c>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>DET0555</t>
+        </is>
+      </c>
+      <c r="H419" t="inlineStr">
+        <is>
+          <t>Stored Office Document Modification by Scripting Host</t>
+        </is>
+      </c>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="J419" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 11, Event ID 1</t>
+        </is>
+      </c>
+      <c r="K419" t="inlineStr">
+        <is>
+          <t>Detects command-line interpreters or scripting hosts creating or modifying business-critical office documents (e.g. .docx, .xlsx, .pdf), which can indicate unauthorized stored data manipulation.</t>
+        </is>
+      </c>
+      <c r="L419" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M419" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N419" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refactor Initial Access tactic rules to support multi-logsource split logic and update Excel tracking
</commit_message>
<xml_diff>
--- a/ocsf_mapped_new_sprint.xlsx
+++ b/ocsf_mapped_new_sprint.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O419"/>
+  <dimension ref="A1:O420"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29296,6 +29296,78 @@
         </is>
       </c>
     </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>AN0320</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>windows</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>initial-access</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>T1566.003</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>Spearphishing via Service</t>
+        </is>
+      </c>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>DET0115</t>
+        </is>
+      </c>
+      <c r="H420" t="inlineStr">
+        <is>
+          <t>Spearphishing via Service - Suspicious Child Process Spawned by Browser or Chat Application</t>
+        </is>
+      </c>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="J420" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1, Event ID 4104</t>
+        </is>
+      </c>
+      <c r="K420" t="inlineStr">
+        <is>
+          <t>Detects suspicious child processes (like cmd.exe, powershell.exe, wscript.exe, rundll32.exe) spawned by web browsers or collaboration/chat applications (Discord, Slack, Telegram, Teams), which indicates browser-initiated exploit execution or user execution of phishing attachments.</t>
+        </is>
+      </c>
+      <c r="L420" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M420" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N420" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refactor lateral-movement rules to support multiple log sources via split rules and update sprint excel tracker
</commit_message>
<xml_diff>
--- a/ocsf_mapped_new_sprint.xlsx
+++ b/ocsf_mapped_new_sprint.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O420"/>
+  <dimension ref="A1:O425"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -576,6 +576,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -648,6 +649,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -720,6 +722,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -792,6 +795,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -864,6 +868,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -936,6 +941,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1008,6 +1014,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1080,6 +1087,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1152,6 +1160,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1224,6 +1233,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1296,6 +1306,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1368,6 +1379,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1440,6 +1452,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1512,6 +1525,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1584,6 +1598,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1656,6 +1671,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1728,6 +1744,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1800,6 +1817,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1872,6 +1890,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1944,6 +1963,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2016,6 +2036,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2088,6 +2109,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2160,6 +2182,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2232,6 +2255,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2304,6 +2328,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2371,6 +2396,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2438,6 +2465,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2505,6 +2534,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2572,6 +2603,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2639,6 +2672,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2706,6 +2741,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2773,6 +2810,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2840,6 +2879,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2907,6 +2948,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2974,6 +3017,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3041,6 +3086,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3113,6 +3160,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3180,6 +3228,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3247,6 +3297,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3314,6 +3366,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3381,6 +3435,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3448,6 +3504,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3515,6 +3573,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3582,6 +3642,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3649,6 +3711,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3716,6 +3780,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3783,6 +3849,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3850,6 +3918,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3917,6 +3987,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3984,6 +4056,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4051,6 +4125,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4118,6 +4194,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4185,6 +4263,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4252,6 +4332,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4319,6 +4401,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4386,6 +4470,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4453,6 +4539,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N58" t="inlineStr"/>
+      <c r="O58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -4520,6 +4608,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4587,6 +4677,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4654,6 +4746,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N61" t="inlineStr"/>
+      <c r="O61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4721,6 +4815,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4788,6 +4884,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N63" t="inlineStr"/>
+      <c r="O63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4855,6 +4953,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4922,6 +5022,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N65" t="inlineStr"/>
+      <c r="O65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4989,6 +5091,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N66" t="inlineStr"/>
+      <c r="O66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5056,6 +5160,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N67" t="inlineStr"/>
+      <c r="O67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -5123,6 +5229,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N68" t="inlineStr"/>
+      <c r="O68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5190,6 +5298,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N69" t="inlineStr"/>
+      <c r="O69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5257,6 +5367,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N70" t="inlineStr"/>
+      <c r="O70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5324,6 +5436,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N71" t="inlineStr"/>
+      <c r="O71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -5391,6 +5505,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N72" t="inlineStr"/>
+      <c r="O72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -5458,6 +5574,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N73" t="inlineStr"/>
+      <c r="O73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -5525,6 +5643,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N74" t="inlineStr"/>
+      <c r="O74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -5592,6 +5712,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N75" t="inlineStr"/>
+      <c r="O75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -5659,6 +5781,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N76" t="inlineStr"/>
+      <c r="O76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -5726,6 +5850,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N77" t="inlineStr"/>
+      <c r="O77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -5793,6 +5919,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N78" t="inlineStr"/>
+      <c r="O78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -5860,6 +5988,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N79" t="inlineStr"/>
+      <c r="O79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -5927,6 +6057,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N80" t="inlineStr"/>
+      <c r="O80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -5994,6 +6126,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N81" t="inlineStr"/>
+      <c r="O81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -6061,6 +6195,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N82" t="inlineStr"/>
+      <c r="O82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -6128,6 +6264,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N83" t="inlineStr"/>
+      <c r="O83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -6195,6 +6333,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N84" t="inlineStr"/>
+      <c r="O84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -6262,6 +6402,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N85" t="inlineStr"/>
+      <c r="O85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -6329,6 +6471,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N86" t="inlineStr"/>
+      <c r="O86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -6396,6 +6540,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N87" t="inlineStr"/>
+      <c r="O87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -6463,6 +6609,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N88" t="inlineStr"/>
+      <c r="O88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -6530,6 +6678,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N89" t="inlineStr"/>
+      <c r="O89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -6597,6 +6747,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N90" t="inlineStr"/>
+      <c r="O90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -6664,6 +6816,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N91" t="inlineStr"/>
+      <c r="O91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -6731,6 +6885,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N92" t="inlineStr"/>
+      <c r="O92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -6798,6 +6954,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N93" t="inlineStr"/>
+      <c r="O93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -6865,6 +7023,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N94" t="inlineStr"/>
+      <c r="O94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -6932,6 +7092,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N95" t="inlineStr"/>
+      <c r="O95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -6999,6 +7161,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N96" t="inlineStr"/>
+      <c r="O96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -7066,6 +7230,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N97" t="inlineStr"/>
+      <c r="O97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -7133,6 +7299,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N98" t="inlineStr"/>
+      <c r="O98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -7200,6 +7368,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N99" t="inlineStr"/>
+      <c r="O99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -7267,6 +7437,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N100" t="inlineStr"/>
+      <c r="O100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -7334,6 +7506,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N101" t="inlineStr"/>
+      <c r="O101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -7401,6 +7575,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N102" t="inlineStr"/>
+      <c r="O102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -7468,6 +7644,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N103" t="inlineStr"/>
+      <c r="O103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -7535,6 +7713,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N104" t="inlineStr"/>
+      <c r="O104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -7602,6 +7782,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N105" t="inlineStr"/>
+      <c r="O105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -7669,6 +7851,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N106" t="inlineStr"/>
+      <c r="O106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -7736,6 +7920,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N107" t="inlineStr"/>
+      <c r="O107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -7803,6 +7989,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N108" t="inlineStr"/>
+      <c r="O108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -7870,6 +8058,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N109" t="inlineStr"/>
+      <c r="O109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -7937,6 +8127,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N110" t="inlineStr"/>
+      <c r="O110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -8009,6 +8201,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -8081,6 +8274,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -8153,6 +8347,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -8225,6 +8420,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -8297,6 +8493,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -8369,6 +8566,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -8441,6 +8639,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -8513,6 +8712,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -8585,6 +8785,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -8657,6 +8858,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -8729,6 +8931,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -8801,6 +9004,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -8873,6 +9077,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -8945,6 +9150,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -9017,6 +9223,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -9089,6 +9296,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -9161,6 +9369,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -9233,6 +9442,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -9300,6 +9510,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N129" t="inlineStr"/>
+      <c r="O129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -9367,6 +9579,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N130" t="inlineStr"/>
+      <c r="O130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -9434,6 +9648,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N131" t="inlineStr"/>
+      <c r="O131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -9501,6 +9717,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N132" t="inlineStr"/>
+      <c r="O132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -9568,6 +9786,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N133" t="inlineStr"/>
+      <c r="O133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -9635,6 +9855,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N134" t="inlineStr"/>
+      <c r="O134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -9702,6 +9924,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N135" t="inlineStr"/>
+      <c r="O135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -9769,6 +9993,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N136" t="inlineStr"/>
+      <c r="O136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -9836,6 +10062,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N137" t="inlineStr"/>
+      <c r="O137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -9903,6 +10131,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N138" t="inlineStr"/>
+      <c r="O138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -9970,6 +10200,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N139" t="inlineStr"/>
+      <c r="O139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -10037,6 +10269,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N140" t="inlineStr"/>
+      <c r="O140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -10104,6 +10338,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N141" t="inlineStr"/>
+      <c r="O141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -10171,6 +10407,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N142" t="inlineStr"/>
+      <c r="O142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -10238,6 +10476,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N143" t="inlineStr"/>
+      <c r="O143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -10305,6 +10545,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N144" t="inlineStr"/>
+      <c r="O144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -10372,6 +10614,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N145" t="inlineStr"/>
+      <c r="O145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -10439,6 +10683,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N146" t="inlineStr"/>
+      <c r="O146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -10506,6 +10752,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N147" t="inlineStr"/>
+      <c r="O147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -10573,6 +10821,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N148" t="inlineStr"/>
+      <c r="O148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -10640,6 +10890,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N149" t="inlineStr"/>
+      <c r="O149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -10707,6 +10959,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N150" t="inlineStr"/>
+      <c r="O150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -10774,6 +11028,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N151" t="inlineStr"/>
+      <c r="O151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -10841,6 +11097,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N152" t="inlineStr"/>
+      <c r="O152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -10908,6 +11166,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N153" t="inlineStr"/>
+      <c r="O153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -10975,6 +11235,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N154" t="inlineStr"/>
+      <c r="O154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -11042,6 +11304,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N155" t="inlineStr"/>
+      <c r="O155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -11109,6 +11373,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N156" t="inlineStr"/>
+      <c r="O156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -11176,6 +11442,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N157" t="inlineStr"/>
+      <c r="O157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -11243,6 +11511,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N158" t="inlineStr"/>
+      <c r="O158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -11310,6 +11580,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N159" t="inlineStr"/>
+      <c r="O159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -11377,6 +11649,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N160" t="inlineStr"/>
+      <c r="O160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -11444,6 +11718,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N161" t="inlineStr"/>
+      <c r="O161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -11511,6 +11787,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N162" t="inlineStr"/>
+      <c r="O162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -11578,6 +11856,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N163" t="inlineStr"/>
+      <c r="O163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -11645,6 +11925,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N164" t="inlineStr"/>
+      <c r="O164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -11712,6 +11994,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N165" t="inlineStr"/>
+      <c r="O165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -11779,6 +12063,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N166" t="inlineStr"/>
+      <c r="O166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -11846,6 +12132,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N167" t="inlineStr"/>
+      <c r="O167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -11913,6 +12201,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N168" t="inlineStr"/>
+      <c r="O168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -11980,6 +12270,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N169" t="inlineStr"/>
+      <c r="O169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -12047,6 +12339,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N170" t="inlineStr"/>
+      <c r="O170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -12114,6 +12408,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N171" t="inlineStr"/>
+      <c r="O171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -12181,6 +12477,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N172" t="inlineStr"/>
+      <c r="O172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -12248,6 +12546,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N173" t="inlineStr"/>
+      <c r="O173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -12315,6 +12615,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N174" t="inlineStr"/>
+      <c r="O174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -12382,6 +12684,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N175" t="inlineStr"/>
+      <c r="O175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -12449,6 +12753,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N176" t="inlineStr"/>
+      <c r="O176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -12516,6 +12822,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N177" t="inlineStr"/>
+      <c r="O177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -12583,6 +12891,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N178" t="inlineStr"/>
+      <c r="O178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -12650,6 +12960,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N179" t="inlineStr"/>
+      <c r="O179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -12717,6 +13029,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N180" t="inlineStr"/>
+      <c r="O180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -12784,6 +13098,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N181" t="inlineStr"/>
+      <c r="O181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -12851,6 +13167,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N182" t="inlineStr"/>
+      <c r="O182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -12918,6 +13236,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N183" t="inlineStr"/>
+      <c r="O183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -12985,6 +13305,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N184" t="inlineStr"/>
+      <c r="O184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -13052,6 +13374,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N185" t="inlineStr"/>
+      <c r="O185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -13119,6 +13443,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N186" t="inlineStr"/>
+      <c r="O186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -13186,6 +13512,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N187" t="inlineStr"/>
+      <c r="O187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -13253,6 +13581,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N188" t="inlineStr"/>
+      <c r="O188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -13320,6 +13650,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N189" t="inlineStr"/>
+      <c r="O189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -13387,6 +13719,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N190" t="inlineStr"/>
+      <c r="O190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -13454,6 +13788,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N191" t="inlineStr"/>
+      <c r="O191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -13521,6 +13857,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N192" t="inlineStr"/>
+      <c r="O192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -13588,6 +13926,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N193" t="inlineStr"/>
+      <c r="O193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -13655,6 +13995,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N194" t="inlineStr"/>
+      <c r="O194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -13722,6 +14064,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N195" t="inlineStr"/>
+      <c r="O195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -13789,6 +14133,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N196" t="inlineStr"/>
+      <c r="O196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -13856,6 +14202,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N197" t="inlineStr"/>
+      <c r="O197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -13923,6 +14271,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N198" t="inlineStr"/>
+      <c r="O198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -13990,6 +14340,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N199" t="inlineStr"/>
+      <c r="O199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -14057,6 +14409,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N200" t="inlineStr"/>
+      <c r="O200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -14124,6 +14478,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N201" t="inlineStr"/>
+      <c r="O201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -14191,6 +14547,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N202" t="inlineStr"/>
+      <c r="O202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -14258,6 +14616,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N203" t="inlineStr"/>
+      <c r="O203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -14325,6 +14685,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N204" t="inlineStr"/>
+      <c r="O204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -14392,6 +14754,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N205" t="inlineStr"/>
+      <c r="O205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -14459,6 +14823,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N206" t="inlineStr"/>
+      <c r="O206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -14526,6 +14892,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N207" t="inlineStr"/>
+      <c r="O207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -14593,6 +14961,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N208" t="inlineStr"/>
+      <c r="O208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -14660,6 +15030,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N209" t="inlineStr"/>
+      <c r="O209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -14727,6 +15099,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N210" t="inlineStr"/>
+      <c r="O210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -14794,6 +15168,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N211" t="inlineStr"/>
+      <c r="O211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -14861,6 +15237,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N212" t="inlineStr"/>
+      <c r="O212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -14928,6 +15306,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N213" t="inlineStr"/>
+      <c r="O213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -14995,6 +15375,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N214" t="inlineStr"/>
+      <c r="O214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -15062,6 +15444,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N215" t="inlineStr"/>
+      <c r="O215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -15129,6 +15513,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N216" t="inlineStr"/>
+      <c r="O216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -15196,6 +15582,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N217" t="inlineStr"/>
+      <c r="O217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -15263,6 +15651,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N218" t="inlineStr"/>
+      <c r="O218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -15330,6 +15720,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N219" t="inlineStr"/>
+      <c r="O219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -15397,6 +15789,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N220" t="inlineStr"/>
+      <c r="O220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -15772,6 +16166,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N225" t="inlineStr"/>
+      <c r="O225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -15839,6 +16235,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N226" t="inlineStr"/>
+      <c r="O226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -15906,6 +16304,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N227" t="inlineStr"/>
+      <c r="O227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -15973,6 +16373,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N228" t="inlineStr"/>
+      <c r="O228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -16040,6 +16442,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N229" t="inlineStr"/>
+      <c r="O229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -16107,6 +16511,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N230" t="inlineStr"/>
+      <c r="O230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -16174,6 +16580,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N231" t="inlineStr"/>
+      <c r="O231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -16241,6 +16649,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N232" t="inlineStr"/>
+      <c r="O232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -16308,6 +16718,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N233" t="inlineStr"/>
+      <c r="O233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -16375,6 +16787,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N234" t="inlineStr"/>
+      <c r="O234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -16442,6 +16856,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N235" t="inlineStr"/>
+      <c r="O235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -16509,6 +16925,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N236" t="inlineStr"/>
+      <c r="O236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -16576,6 +16994,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N237" t="inlineStr"/>
+      <c r="O237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -16643,6 +17063,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N238" t="inlineStr"/>
+      <c r="O238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -16710,6 +17132,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N239" t="inlineStr"/>
+      <c r="O239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -16777,6 +17201,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N240" t="inlineStr"/>
+      <c r="O240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -16844,6 +17270,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N241" t="inlineStr"/>
+      <c r="O241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -16911,6 +17339,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N242" t="inlineStr"/>
+      <c r="O242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -16978,6 +17408,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N243" t="inlineStr"/>
+      <c r="O243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -17045,6 +17477,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N244" t="inlineStr"/>
+      <c r="O244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -17112,6 +17546,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N245" t="inlineStr"/>
+      <c r="O245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -17179,6 +17615,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N246" t="inlineStr"/>
+      <c r="O246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -17246,6 +17684,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N247" t="inlineStr"/>
+      <c r="O247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -17313,6 +17753,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N248" t="inlineStr"/>
+      <c r="O248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -17380,6 +17822,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N249" t="inlineStr"/>
+      <c r="O249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -17447,6 +17891,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N250" t="inlineStr"/>
+      <c r="O250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -17514,6 +17960,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N251" t="inlineStr"/>
+      <c r="O251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -17581,6 +18029,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N252" t="inlineStr"/>
+      <c r="O252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -17648,6 +18098,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N253" t="inlineStr"/>
+      <c r="O253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -17715,6 +18167,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N254" t="inlineStr"/>
+      <c r="O254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -17782,6 +18236,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N255" t="inlineStr"/>
+      <c r="O255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -17849,6 +18305,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N256" t="inlineStr"/>
+      <c r="O256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -17916,6 +18374,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N257" t="inlineStr"/>
+      <c r="O257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -17983,6 +18443,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N258" t="inlineStr"/>
+      <c r="O258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -18050,6 +18512,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N259" t="inlineStr"/>
+      <c r="O259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -18117,6 +18581,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N260" t="inlineStr"/>
+      <c r="O260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -18184,6 +18650,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N261" t="inlineStr"/>
+      <c r="O261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -18251,6 +18719,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N262" t="inlineStr"/>
+      <c r="O262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -18318,6 +18788,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N263" t="inlineStr"/>
+      <c r="O263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -18385,6 +18857,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N264" t="inlineStr"/>
+      <c r="O264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -18452,6 +18926,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N265" t="inlineStr"/>
+      <c r="O265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -18519,6 +18995,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N266" t="inlineStr"/>
+      <c r="O266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -18586,6 +19064,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N267" t="inlineStr"/>
+      <c r="O267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -18653,6 +19133,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N268" t="inlineStr"/>
+      <c r="O268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -18720,6 +19202,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N269" t="inlineStr"/>
+      <c r="O269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -18787,6 +19271,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N270" t="inlineStr"/>
+      <c r="O270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -18854,6 +19340,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N271" t="inlineStr"/>
+      <c r="O271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -18921,6 +19409,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N272" t="inlineStr"/>
+      <c r="O272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -18988,6 +19478,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N273" t="inlineStr"/>
+      <c r="O273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -19055,6 +19547,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N274" t="inlineStr"/>
+      <c r="O274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -19122,6 +19616,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N275" t="inlineStr"/>
+      <c r="O275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -19189,6 +19685,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N276" t="inlineStr"/>
+      <c r="O276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -19256,6 +19754,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N277" t="inlineStr"/>
+      <c r="O277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -19323,6 +19823,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N278" t="inlineStr"/>
+      <c r="O278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -19472,6 +19974,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -19544,6 +20047,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O281" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -19616,6 +20120,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -19688,6 +20193,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -19760,6 +20266,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O284" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -19832,6 +20339,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O285" t="inlineStr"/>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -19904,6 +20412,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O286" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -19976,6 +20485,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O287" t="inlineStr"/>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -20048,6 +20558,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O288" t="inlineStr"/>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -20120,6 +20631,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O289" t="inlineStr"/>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -20192,6 +20704,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O290" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -20264,6 +20777,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O291" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -20336,6 +20850,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O292" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -20408,6 +20923,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O293" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -20480,6 +20996,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O294" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -20552,6 +21069,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -20624,6 +21142,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O296" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -20696,6 +21215,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O297" t="inlineStr"/>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -20768,6 +21288,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O298" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -20840,6 +21361,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O299" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -20912,6 +21434,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O300" t="inlineStr"/>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -20984,6 +21507,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O301" t="inlineStr"/>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -21056,6 +21580,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O302" t="inlineStr"/>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -21128,6 +21653,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O303" t="inlineStr"/>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -21200,6 +21726,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O304" t="inlineStr"/>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -21272,6 +21799,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O305" t="inlineStr"/>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -21339,6 +21867,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N306" t="inlineStr"/>
+      <c r="O306" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -21406,6 +21936,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N307" t="inlineStr"/>
+      <c r="O307" t="inlineStr"/>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -21473,6 +22005,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N308" t="inlineStr"/>
+      <c r="O308" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -21540,6 +22074,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N309" t="inlineStr"/>
+      <c r="O309" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -21607,6 +22143,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N310" t="inlineStr"/>
+      <c r="O310" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -21674,6 +22212,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N311" t="inlineStr"/>
+      <c r="O311" t="inlineStr"/>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -21741,6 +22281,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N312" t="inlineStr"/>
+      <c r="O312" t="inlineStr"/>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -21808,6 +22350,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N313" t="inlineStr"/>
+      <c r="O313" t="inlineStr"/>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -21875,6 +22419,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N314" t="inlineStr"/>
+      <c r="O314" t="inlineStr"/>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -21942,6 +22488,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N315" t="inlineStr"/>
+      <c r="O315" t="inlineStr"/>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -22009,6 +22557,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N316" t="inlineStr"/>
+      <c r="O316" t="inlineStr"/>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -22076,6 +22626,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N317" t="inlineStr"/>
+      <c r="O317" t="inlineStr"/>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -22143,6 +22695,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N318" t="inlineStr"/>
+      <c r="O318" t="inlineStr"/>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -22210,6 +22764,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N319" t="inlineStr"/>
+      <c r="O319" t="inlineStr"/>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -22277,6 +22833,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N320" t="inlineStr"/>
+      <c r="O320" t="inlineStr"/>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -22344,6 +22902,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N321" t="inlineStr"/>
+      <c r="O321" t="inlineStr"/>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -22411,6 +22971,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N322" t="inlineStr"/>
+      <c r="O322" t="inlineStr"/>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -22478,6 +23040,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N323" t="inlineStr"/>
+      <c r="O323" t="inlineStr"/>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -22545,6 +23109,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N324" t="inlineStr"/>
+      <c r="O324" t="inlineStr"/>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -22612,6 +23178,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N325" t="inlineStr"/>
+      <c r="O325" t="inlineStr"/>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -22679,6 +23247,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N326" t="inlineStr"/>
+      <c r="O326" t="inlineStr"/>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -22746,6 +23316,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N327" t="inlineStr"/>
+      <c r="O327" t="inlineStr"/>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -22813,6 +23385,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N328" t="inlineStr"/>
+      <c r="O328" t="inlineStr"/>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -22880,6 +23454,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N329" t="inlineStr"/>
+      <c r="O329" t="inlineStr"/>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -22947,6 +23523,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N330" t="inlineStr"/>
+      <c r="O330" t="inlineStr"/>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -23014,6 +23592,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N331" t="inlineStr"/>
+      <c r="O331" t="inlineStr"/>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -23081,6 +23661,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N332" t="inlineStr"/>
+      <c r="O332" t="inlineStr"/>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -23148,6 +23730,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N333" t="inlineStr"/>
+      <c r="O333" t="inlineStr"/>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -23215,6 +23799,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N334" t="inlineStr"/>
+      <c r="O334" t="inlineStr"/>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -23282,6 +23868,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N335" t="inlineStr"/>
+      <c r="O335" t="inlineStr"/>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -23349,6 +23937,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N336" t="inlineStr"/>
+      <c r="O336" t="inlineStr"/>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -23421,6 +24011,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O337" t="inlineStr"/>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -23493,6 +24084,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O338" t="inlineStr"/>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -23565,6 +24157,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O339" t="inlineStr"/>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -23637,6 +24230,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O340" t="inlineStr"/>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -23709,6 +24303,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O341" t="inlineStr"/>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -23781,6 +24376,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O342" t="inlineStr"/>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -23853,6 +24449,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O343" t="inlineStr"/>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -23920,6 +24517,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N344" t="inlineStr"/>
+      <c r="O344" t="inlineStr"/>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -23987,6 +24586,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N345" t="inlineStr"/>
+      <c r="O345" t="inlineStr"/>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -24054,6 +24655,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N346" t="inlineStr"/>
+      <c r="O346" t="inlineStr"/>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -24121,6 +24724,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N347" t="inlineStr"/>
+      <c r="O347" t="inlineStr"/>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -24188,6 +24793,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N348" t="inlineStr"/>
+      <c r="O348" t="inlineStr"/>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -24255,6 +24862,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N349" t="inlineStr"/>
+      <c r="O349" t="inlineStr"/>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -24322,6 +24931,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N350" t="inlineStr"/>
+      <c r="O350" t="inlineStr"/>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -24389,6 +25000,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N351" t="inlineStr"/>
+      <c r="O351" t="inlineStr"/>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -24456,6 +25069,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N352" t="inlineStr"/>
+      <c r="O352" t="inlineStr"/>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
@@ -24523,6 +25138,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N353" t="inlineStr"/>
+      <c r="O353" t="inlineStr"/>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -24590,6 +25207,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N354" t="inlineStr"/>
+      <c r="O354" t="inlineStr"/>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -24657,6 +25276,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N355" t="inlineStr"/>
+      <c r="O355" t="inlineStr"/>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -24724,6 +25345,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N356" t="inlineStr"/>
+      <c r="O356" t="inlineStr"/>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -24791,6 +25414,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N357" t="inlineStr"/>
+      <c r="O357" t="inlineStr"/>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -24858,6 +25483,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N358" t="inlineStr"/>
+      <c r="O358" t="inlineStr"/>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -24925,6 +25552,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N359" t="inlineStr"/>
+      <c r="O359" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -24992,6 +25621,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N360" t="inlineStr"/>
+      <c r="O360" t="inlineStr"/>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -25059,6 +25690,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N361" t="inlineStr"/>
+      <c r="O361" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -25126,6 +25759,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N362" t="inlineStr"/>
+      <c r="O362" t="inlineStr"/>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -25193,6 +25828,8 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N363" t="inlineStr"/>
+      <c r="O363" t="inlineStr"/>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -25265,6 +25902,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O364" t="inlineStr"/>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -25337,6 +25975,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O365" t="inlineStr"/>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -25409,6 +26048,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O366" t="inlineStr"/>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -25481,6 +26121,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O367" t="inlineStr"/>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -25553,6 +26194,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O368" t="inlineStr"/>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -25625,6 +26267,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O369" t="inlineStr"/>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
@@ -25697,6 +26340,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O370" t="inlineStr"/>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
@@ -25769,6 +26413,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O371" t="inlineStr"/>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
@@ -25841,6 +26486,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O372" t="inlineStr"/>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
@@ -25913,6 +26559,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O373" t="inlineStr"/>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
@@ -25985,6 +26632,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O374" t="inlineStr"/>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
@@ -26057,6 +26705,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O375" t="inlineStr"/>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
@@ -26129,6 +26778,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O376" t="inlineStr"/>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
@@ -27279,6 +27929,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O391" t="inlineStr"/>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
@@ -27351,6 +28002,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O392" t="inlineStr"/>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
@@ -27423,6 +28075,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O393" t="inlineStr"/>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
@@ -27495,6 +28148,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O394" t="inlineStr"/>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
@@ -27567,6 +28221,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O395" t="inlineStr"/>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
@@ -27639,6 +28294,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O396" t="inlineStr"/>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
@@ -27711,6 +28367,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O397" t="inlineStr"/>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
@@ -27783,6 +28440,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O398" t="inlineStr"/>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
@@ -27855,6 +28513,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O399" t="inlineStr"/>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
@@ -27927,6 +28586,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O400" t="inlineStr"/>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
@@ -27999,6 +28659,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O401" t="inlineStr"/>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
@@ -28071,6 +28732,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O402" t="inlineStr"/>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
@@ -28143,6 +28805,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O403" t="inlineStr"/>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
@@ -28215,6 +28878,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O404" t="inlineStr"/>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
@@ -28287,6 +28951,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O405" t="inlineStr"/>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
@@ -28359,6 +29024,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O406" t="inlineStr"/>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
@@ -28431,6 +29097,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O407" t="inlineStr"/>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
@@ -28503,6 +29170,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O408" t="inlineStr"/>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
@@ -28550,11 +29218,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="J409" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="J409" t="inlineStr"/>
       <c r="K409" t="inlineStr">
         <is>
           <t>This technique is not detectable from Sysmon, Windows Security, or Defender logs.</t>
@@ -28575,6 +29239,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O409" t="inlineStr"/>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
@@ -28647,6 +29312,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O410" t="inlineStr"/>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
@@ -28719,6 +29385,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O411" t="inlineStr"/>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
@@ -28791,6 +29458,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O412" t="inlineStr"/>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
@@ -28863,6 +29531,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O413" t="inlineStr"/>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
@@ -28935,6 +29604,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O414" t="inlineStr"/>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
@@ -29007,6 +29677,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O415" t="inlineStr"/>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
@@ -29079,6 +29750,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O416" t="inlineStr"/>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
@@ -29151,6 +29823,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O417" t="inlineStr"/>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
@@ -29223,6 +29896,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O418" t="inlineStr"/>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
@@ -29295,6 +29969,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O419" t="inlineStr"/>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
@@ -29367,6 +30042,372 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O420" t="inlineStr"/>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>AN0216</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>lateral-movement</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>T1563</t>
+        </is>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>Remote Service Session Hijacking</t>
+        </is>
+      </c>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t>DET0079</t>
+        </is>
+      </c>
+      <c r="H421" t="inlineStr">
+        <is>
+          <t>Detection of Remote Service Session Hijacking</t>
+        </is>
+      </c>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t>host-local feeds only</t>
+        </is>
+      </c>
+      <c r="J421" t="inlineStr">
+        <is>
+          <t>WinEventLog:Security; WinEventLog:Sysmon</t>
+        </is>
+      </c>
+      <c r="K421" t="inlineStr">
+        <is>
+          <t>Detects RDP session hijacking via tscon.exe executed under SYSTEM context or via sc.exe creating a service with tscon in the binary path. Adversaries with SYSTEM privileges use this native Windows utility to take control of disconnected RDP sessions without requiring credentials (T1563.002).</t>
+        </is>
+      </c>
+      <c r="L421" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M421" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N421" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O421" t="inlineStr"/>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>AN0516</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>lateral-movement</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>T1570</t>
+        </is>
+      </c>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t>Lateral Tool Transfer</t>
+        </is>
+      </c>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t>DET0183</t>
+        </is>
+      </c>
+      <c r="H422" t="inlineStr">
+        <is>
+          <t>Detection Strategy for Lateral Tool Transfer across OS platforms</t>
+        </is>
+      </c>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t>host-local feeds only</t>
+        </is>
+      </c>
+      <c r="J422" t="inlineStr">
+        <is>
+          <t>WinEventLog:Security; WinEventLog:Sysmon</t>
+        </is>
+      </c>
+      <c r="K422" t="inlineStr">
+        <is>
+          <t>Detects command-line copy or file transfer utilities (copy, move, xcopy, robocopy) targeting administrative shares (e.g. C$, ADMIN$), which can indicate lateral tool transfer.</t>
+        </is>
+      </c>
+      <c r="L422" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M422" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N422" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O422" t="inlineStr"/>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>AN0954</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>lateral-movement</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>T1550</t>
+        </is>
+      </c>
+      <c r="F423" t="inlineStr">
+        <is>
+          <t>Use Alternate Authentication Material</t>
+        </is>
+      </c>
+      <c r="G423" t="inlineStr">
+        <is>
+          <t>DET0338</t>
+        </is>
+      </c>
+      <c r="H423" t="inlineStr">
+        <is>
+          <t>Behavioral Detection Strategy for Use Alternate Authentication Material (T1550)</t>
+        </is>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t>host-local feeds only</t>
+        </is>
+      </c>
+      <c r="J423" t="inlineStr">
+        <is>
+          <t>WinEventLog:Security; WinEventLog:Sysmon</t>
+        </is>
+      </c>
+      <c r="K423" t="inlineStr">
+        <is>
+          <t>Detects successful authentication events utilizing logon type 9 (NewCredentials), which is generated when alternate credentials are used for outbound authentication (e.g. Pass-the-Hash or Pass-the-Ticket).</t>
+        </is>
+      </c>
+      <c r="L423" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M423" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N423" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O423" t="inlineStr"/>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>AN1298</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>lateral-movement</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>T1080</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>Taint Shared Content</t>
+        </is>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>DET0471</t>
+        </is>
+      </c>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t>Detection of Tainted Content Written to Shared Storage</t>
+        </is>
+      </c>
+      <c r="I424" t="inlineStr">
+        <is>
+          <t>host-local feeds only</t>
+        </is>
+      </c>
+      <c r="J424" t="inlineStr">
+        <is>
+          <t>WinEventLog:Security; WinEventLog:Sysmon</t>
+        </is>
+      </c>
+      <c r="K424" t="inlineStr">
+        <is>
+          <t>Detects file creation events dropping executable, scripting, or shortcut extensions (e.g., .exe, .vbs, .lnk) onto administrative network shared directory paths.</t>
+        </is>
+      </c>
+      <c r="L424" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M424" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N424" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O424" t="inlineStr"/>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>AN1620</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>Endpoint-offline</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>lateral-movement</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>T1563.002</t>
+        </is>
+      </c>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t>Remote Service Session Hijacking: RDP Hijacking</t>
+        </is>
+      </c>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t>DET0588</t>
+        </is>
+      </c>
+      <c r="H425" t="inlineStr">
+        <is>
+          <t>Detection of Remote Service Session Hijacking for RDP.</t>
+        </is>
+      </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t>host-local feeds only</t>
+        </is>
+      </c>
+      <c r="J425" t="inlineStr">
+        <is>
+          <t>WinEventLog:Security; WinEventLog:Sysmon</t>
+        </is>
+      </c>
+      <c r="K425" t="inlineStr">
+        <is>
+          <t>Detects RDP session hijacking attempts using the native Windows tscon.exe utility, which transfers an active terminal session to a different destination session.</t>
+        </is>
+      </c>
+      <c r="L425" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M425" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N425" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O425" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Refactor defense-impairment rules to support multiple log sources via split rules and update sprint excel tracker
</commit_message>
<xml_diff>
--- a/ocsf_mapped_new_sprint.xlsx
+++ b/ocsf_mapped_new_sprint.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O425"/>
+  <dimension ref="A1:O434"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30409,6 +30409,375 @@
       </c>
       <c r="O425" t="inlineStr"/>
     </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>AN0153</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr"/>
+      <c r="C426" t="inlineStr"/>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>defense-impairment</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>T1553.004</t>
+        </is>
+      </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t>Install Root Certificate</t>
+        </is>
+      </c>
+      <c r="G426" t="inlineStr"/>
+      <c r="H426" t="inlineStr"/>
+      <c r="I426" t="inlineStr"/>
+      <c r="J426" t="inlineStr"/>
+      <c r="K426" t="inlineStr"/>
+      <c r="L426" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M426" t="inlineStr"/>
+      <c r="N426" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O426" t="inlineStr"/>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>AN0323</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr"/>
+      <c r="C427" t="inlineStr"/>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>defense-impairment</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>T1688</t>
+        </is>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>Disable or Modify Security Tools</t>
+        </is>
+      </c>
+      <c r="G427" t="inlineStr"/>
+      <c r="H427" t="inlineStr"/>
+      <c r="I427" t="inlineStr"/>
+      <c r="J427" t="inlineStr"/>
+      <c r="K427" t="inlineStr"/>
+      <c r="L427" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M427" t="inlineStr"/>
+      <c r="N427" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O427" t="inlineStr"/>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>AN0406</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr"/>
+      <c r="C428" t="inlineStr"/>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>defense-impairment</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>T1686</t>
+        </is>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>Disable Windows Defender Real-time Protection</t>
+        </is>
+      </c>
+      <c r="G428" t="inlineStr"/>
+      <c r="H428" t="inlineStr"/>
+      <c r="I428" t="inlineStr"/>
+      <c r="J428" t="inlineStr"/>
+      <c r="K428" t="inlineStr"/>
+      <c r="L428" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M428" t="inlineStr"/>
+      <c r="N428" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O428" t="inlineStr"/>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>AN0535</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr"/>
+      <c r="C429" t="inlineStr"/>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>defense-impairment</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>T1685.001</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>Disable UAC via Registry</t>
+        </is>
+      </c>
+      <c r="G429" t="inlineStr"/>
+      <c r="H429" t="inlineStr"/>
+      <c r="I429" t="inlineStr"/>
+      <c r="J429" t="inlineStr"/>
+      <c r="K429" t="inlineStr"/>
+      <c r="L429" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M429" t="inlineStr"/>
+      <c r="N429" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O429" t="inlineStr"/>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>AN0643</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr"/>
+      <c r="C430" t="inlineStr"/>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>defense-impairment</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>T1553.002</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t>Bypass SmartScreen via Zone.Identifier</t>
+        </is>
+      </c>
+      <c r="G430" t="inlineStr"/>
+      <c r="H430" t="inlineStr"/>
+      <c r="I430" t="inlineStr"/>
+      <c r="J430" t="inlineStr"/>
+      <c r="K430" t="inlineStr"/>
+      <c r="L430" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M430" t="inlineStr"/>
+      <c r="N430" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O430" t="inlineStr"/>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>AN0755</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr"/>
+      <c r="C431" t="inlineStr"/>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>defense-impairment</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>T1484</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>Disable Windows Firewall via Netsh</t>
+        </is>
+      </c>
+      <c r="G431" t="inlineStr"/>
+      <c r="H431" t="inlineStr"/>
+      <c r="I431" t="inlineStr"/>
+      <c r="J431" t="inlineStr"/>
+      <c r="K431" t="inlineStr"/>
+      <c r="L431" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M431" t="inlineStr"/>
+      <c r="N431" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O431" t="inlineStr"/>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>AN0781</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr"/>
+      <c r="C432" t="inlineStr"/>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>defense-impairment</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>T1112</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>Modify Registry to Impair Security</t>
+        </is>
+      </c>
+      <c r="G432" t="inlineStr"/>
+      <c r="H432" t="inlineStr"/>
+      <c r="I432" t="inlineStr"/>
+      <c r="J432" t="inlineStr"/>
+      <c r="K432" t="inlineStr"/>
+      <c r="L432" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M432" t="inlineStr"/>
+      <c r="N432" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O432" t="inlineStr"/>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>AN0834</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr"/>
+      <c r="C433" t="inlineStr"/>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>defense-impairment</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>T1222</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>Impair Defenses - Modify File Permissions</t>
+        </is>
+      </c>
+      <c r="G433" t="inlineStr"/>
+      <c r="H433" t="inlineStr"/>
+      <c r="I433" t="inlineStr"/>
+      <c r="J433" t="inlineStr"/>
+      <c r="K433" t="inlineStr"/>
+      <c r="L433" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M433" t="inlineStr"/>
+      <c r="N433" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O433" t="inlineStr"/>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>AN0854</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr"/>
+      <c r="C434" t="inlineStr"/>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>defense-impairment</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>T1484.001</t>
+        </is>
+      </c>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t>Disable Group Policy Updates</t>
+        </is>
+      </c>
+      <c r="G434" t="inlineStr"/>
+      <c r="H434" t="inlineStr"/>
+      <c r="I434" t="inlineStr"/>
+      <c r="J434" t="inlineStr"/>
+      <c r="K434" t="inlineStr"/>
+      <c r="L434" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M434" t="inlineStr"/>
+      <c r="N434" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O434" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refactor execution rules to multiple log sources (split rules) and update tracking workbook
</commit_message>
<xml_diff>
--- a/ocsf_mapped_new_sprint.xlsx
+++ b/ocsf_mapped_new_sprint.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O434"/>
+  <dimension ref="A1:O444"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30778,6 +30778,416 @@
       </c>
       <c r="O434" t="inlineStr"/>
     </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>AN0009</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr"/>
+      <c r="C435" t="inlineStr"/>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>execution</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>T1574.007</t>
+        </is>
+      </c>
+      <c r="F435" t="inlineStr">
+        <is>
+          <t>Hijack Execution Flow: Path Abuse</t>
+        </is>
+      </c>
+      <c r="G435" t="inlineStr"/>
+      <c r="H435" t="inlineStr"/>
+      <c r="I435" t="inlineStr"/>
+      <c r="J435" t="inlineStr"/>
+      <c r="K435" t="inlineStr"/>
+      <c r="L435" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M435" t="inlineStr"/>
+      <c r="N435" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O435" t="inlineStr"/>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>AN0052</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr"/>
+      <c r="C436" t="inlineStr"/>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>execution</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>T1129</t>
+        </is>
+      </c>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>Shared Modules</t>
+        </is>
+      </c>
+      <c r="G436" t="inlineStr"/>
+      <c r="H436" t="inlineStr"/>
+      <c r="I436" t="inlineStr"/>
+      <c r="J436" t="inlineStr"/>
+      <c r="K436" t="inlineStr"/>
+      <c r="L436" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M436" t="inlineStr"/>
+      <c r="N436" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O436" t="inlineStr"/>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>AN0108</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr"/>
+      <c r="C437" t="inlineStr"/>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>execution</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>T1574.005</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>Hijack Execution Flow: DLL Search Order Hijacking</t>
+        </is>
+      </c>
+      <c r="G437" t="inlineStr"/>
+      <c r="H437" t="inlineStr"/>
+      <c r="I437" t="inlineStr"/>
+      <c r="J437" t="inlineStr"/>
+      <c r="K437" t="inlineStr"/>
+      <c r="L437" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M437" t="inlineStr"/>
+      <c r="N437" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O437" t="inlineStr"/>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>AN0176</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr"/>
+      <c r="C438" t="inlineStr"/>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>execution</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>T1574.009</t>
+        </is>
+      </c>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>Hijack Execution Flow: Path Hijacking</t>
+        </is>
+      </c>
+      <c r="G438" t="inlineStr"/>
+      <c r="H438" t="inlineStr"/>
+      <c r="I438" t="inlineStr"/>
+      <c r="J438" t="inlineStr"/>
+      <c r="K438" t="inlineStr"/>
+      <c r="L438" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M438" t="inlineStr"/>
+      <c r="N438" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O438" t="inlineStr"/>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>AN0209</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr"/>
+      <c r="C439" t="inlineStr"/>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>execution</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>T1059.005</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>Command and Scripting Interpreter: VBScript</t>
+        </is>
+      </c>
+      <c r="G439" t="inlineStr"/>
+      <c r="H439" t="inlineStr"/>
+      <c r="I439" t="inlineStr"/>
+      <c r="J439" t="inlineStr"/>
+      <c r="K439" t="inlineStr"/>
+      <c r="L439" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M439" t="inlineStr"/>
+      <c r="N439" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O439" t="inlineStr"/>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>AN0258</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr"/>
+      <c r="C440" t="inlineStr"/>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>execution</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>T1053</t>
+        </is>
+      </c>
+      <c r="F440" t="inlineStr">
+        <is>
+          <t>Scheduled Task/Job</t>
+        </is>
+      </c>
+      <c r="G440" t="inlineStr"/>
+      <c r="H440" t="inlineStr"/>
+      <c r="I440" t="inlineStr"/>
+      <c r="J440" t="inlineStr"/>
+      <c r="K440" t="inlineStr"/>
+      <c r="L440" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M440" t="inlineStr"/>
+      <c r="N440" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O440" t="inlineStr"/>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>AN0278</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr"/>
+      <c r="C441" t="inlineStr"/>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>execution</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>T1059.011</t>
+        </is>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>Command and Scripting Interpreter: JavaScript</t>
+        </is>
+      </c>
+      <c r="G441" t="inlineStr"/>
+      <c r="H441" t="inlineStr"/>
+      <c r="I441" t="inlineStr"/>
+      <c r="J441" t="inlineStr"/>
+      <c r="K441" t="inlineStr"/>
+      <c r="L441" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M441" t="inlineStr"/>
+      <c r="N441" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O441" t="inlineStr"/>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>AN0550</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr"/>
+      <c r="C442" t="inlineStr"/>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>execution</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>T1127.002</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>Trusted Developer Utilities Proxy Execution: MSBuild</t>
+        </is>
+      </c>
+      <c r="G442" t="inlineStr"/>
+      <c r="H442" t="inlineStr"/>
+      <c r="I442" t="inlineStr"/>
+      <c r="J442" t="inlineStr"/>
+      <c r="K442" t="inlineStr"/>
+      <c r="L442" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M442" t="inlineStr"/>
+      <c r="N442" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O442" t="inlineStr"/>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>AN0577</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr"/>
+      <c r="C443" t="inlineStr"/>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>execution</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>T1574.001</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr">
+        <is>
+          <t>Hijack Execution Flow: DLL Side-Loading</t>
+        </is>
+      </c>
+      <c r="G443" t="inlineStr"/>
+      <c r="H443" t="inlineStr"/>
+      <c r="I443" t="inlineStr"/>
+      <c r="J443" t="inlineStr"/>
+      <c r="K443" t="inlineStr"/>
+      <c r="L443" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M443" t="inlineStr"/>
+      <c r="N443" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O443" t="inlineStr"/>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>AN0609</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr"/>
+      <c r="C444" t="inlineStr"/>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>execution</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>T1574</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t>Hijack Execution Flow</t>
+        </is>
+      </c>
+      <c r="G444" t="inlineStr"/>
+      <c r="H444" t="inlineStr"/>
+      <c r="I444" t="inlineStr"/>
+      <c r="J444" t="inlineStr"/>
+      <c r="K444" t="inlineStr"/>
+      <c r="L444" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M444" t="inlineStr"/>
+      <c r="N444" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O444" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refactor 10 exfiltration rules to support multiple log sources via split rules and update tracking workbook
</commit_message>
<xml_diff>
--- a/ocsf_mapped_new_sprint.xlsx
+++ b/ocsf_mapped_new_sprint.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O444"/>
+  <dimension ref="A1:O454"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31188,6 +31188,416 @@
       </c>
       <c r="O444" t="inlineStr"/>
     </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>AN0212</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr"/>
+      <c r="C445" t="inlineStr"/>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>exfiltration</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>T1011</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t>Exfiltration Over Other Network Medium</t>
+        </is>
+      </c>
+      <c r="G445" t="inlineStr"/>
+      <c r="H445" t="inlineStr"/>
+      <c r="I445" t="inlineStr"/>
+      <c r="J445" t="inlineStr"/>
+      <c r="K445" t="inlineStr"/>
+      <c r="L445" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M445" t="inlineStr"/>
+      <c r="N445" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O445" t="inlineStr"/>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>AN0342</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr"/>
+      <c r="C446" t="inlineStr"/>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>exfiltration</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>T1052</t>
+        </is>
+      </c>
+      <c r="F446" t="inlineStr">
+        <is>
+          <t>Exfiltration Over Physical Medium</t>
+        </is>
+      </c>
+      <c r="G446" t="inlineStr"/>
+      <c r="H446" t="inlineStr"/>
+      <c r="I446" t="inlineStr"/>
+      <c r="J446" t="inlineStr"/>
+      <c r="K446" t="inlineStr"/>
+      <c r="L446" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M446" t="inlineStr"/>
+      <c r="N446" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O446" t="inlineStr"/>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>AN0367</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr"/>
+      <c r="C447" t="inlineStr"/>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>exfiltration</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>T1048</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t>Exfiltration Over Alternative Protocol</t>
+        </is>
+      </c>
+      <c r="G447" t="inlineStr"/>
+      <c r="H447" t="inlineStr"/>
+      <c r="I447" t="inlineStr"/>
+      <c r="J447" t="inlineStr"/>
+      <c r="K447" t="inlineStr"/>
+      <c r="L447" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M447" t="inlineStr"/>
+      <c r="N447" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O447" t="inlineStr"/>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>AN0436</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr"/>
+      <c r="C448" t="inlineStr"/>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>exfiltration</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>T1567.004</t>
+        </is>
+      </c>
+      <c r="F448" t="inlineStr">
+        <is>
+          <t>Exfiltration Over Web Service: Exfiltration to Cloud Storage</t>
+        </is>
+      </c>
+      <c r="G448" t="inlineStr"/>
+      <c r="H448" t="inlineStr"/>
+      <c r="I448" t="inlineStr"/>
+      <c r="J448" t="inlineStr"/>
+      <c r="K448" t="inlineStr"/>
+      <c r="L448" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M448" t="inlineStr"/>
+      <c r="N448" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O448" t="inlineStr"/>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>AN0616</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr"/>
+      <c r="C449" t="inlineStr"/>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>exfiltration</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>T1052.001</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t>Exfiltration Over Physical Medium: Exfiltration over USB</t>
+        </is>
+      </c>
+      <c r="G449" t="inlineStr"/>
+      <c r="H449" t="inlineStr"/>
+      <c r="I449" t="inlineStr"/>
+      <c r="J449" t="inlineStr"/>
+      <c r="K449" t="inlineStr"/>
+      <c r="L449" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M449" t="inlineStr"/>
+      <c r="N449" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O449" t="inlineStr"/>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>AN0787</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr"/>
+      <c r="C450" t="inlineStr"/>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>exfiltration</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>T1567.003</t>
+        </is>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t>Exfiltration Over Web Service: Exfiltration to Code Repository</t>
+        </is>
+      </c>
+      <c r="G450" t="inlineStr"/>
+      <c r="H450" t="inlineStr"/>
+      <c r="I450" t="inlineStr"/>
+      <c r="J450" t="inlineStr"/>
+      <c r="K450" t="inlineStr"/>
+      <c r="L450" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M450" t="inlineStr"/>
+      <c r="N450" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O450" t="inlineStr"/>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>AN0895</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr"/>
+      <c r="C451" t="inlineStr"/>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>exfiltration</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>T1567.001</t>
+        </is>
+      </c>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>Exfiltration Over Web Service: Exfiltration to Webhook</t>
+        </is>
+      </c>
+      <c r="G451" t="inlineStr"/>
+      <c r="H451" t="inlineStr"/>
+      <c r="I451" t="inlineStr"/>
+      <c r="J451" t="inlineStr"/>
+      <c r="K451" t="inlineStr"/>
+      <c r="L451" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M451" t="inlineStr"/>
+      <c r="N451" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O451" t="inlineStr"/>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>AN1113</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr"/>
+      <c r="C452" t="inlineStr"/>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>exfiltration</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>T1020</t>
+        </is>
+      </c>
+      <c r="F452" t="inlineStr">
+        <is>
+          <t>Automated Exfiltration</t>
+        </is>
+      </c>
+      <c r="G452" t="inlineStr"/>
+      <c r="H452" t="inlineStr"/>
+      <c r="I452" t="inlineStr"/>
+      <c r="J452" t="inlineStr"/>
+      <c r="K452" t="inlineStr"/>
+      <c r="L452" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M452" t="inlineStr"/>
+      <c r="N452" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O452" t="inlineStr"/>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>AN1118</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr"/>
+      <c r="C453" t="inlineStr"/>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>exfiltration</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>T1029</t>
+        </is>
+      </c>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>Scheduled Transfer</t>
+        </is>
+      </c>
+      <c r="G453" t="inlineStr"/>
+      <c r="H453" t="inlineStr"/>
+      <c r="I453" t="inlineStr"/>
+      <c r="J453" t="inlineStr"/>
+      <c r="K453" t="inlineStr"/>
+      <c r="L453" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M453" t="inlineStr"/>
+      <c r="N453" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O453" t="inlineStr"/>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>AN1389</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr"/>
+      <c r="C454" t="inlineStr"/>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>exfiltration</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>T1048.001</t>
+        </is>
+      </c>
+      <c r="F454" t="inlineStr">
+        <is>
+          <t>Exfiltration Over Alternative Protocol: Symmetric Cryptography</t>
+        </is>
+      </c>
+      <c r="G454" t="inlineStr"/>
+      <c r="H454" t="inlineStr"/>
+      <c r="I454" t="inlineStr"/>
+      <c r="J454" t="inlineStr"/>
+      <c r="K454" t="inlineStr"/>
+      <c r="L454" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M454" t="inlineStr"/>
+      <c r="N454" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O454" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refactor collection and persistence rules for multi-source log support
</commit_message>
<xml_diff>
--- a/ocsf_mapped_new_sprint.xlsx
+++ b/ocsf_mapped_new_sprint.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O454"/>
+  <dimension ref="A1:O463"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31598,6 +31598,375 @@
       </c>
       <c r="O454" t="inlineStr"/>
     </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>AN0040</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr"/>
+      <c r="C455" t="inlineStr"/>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>collection</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>T1074</t>
+        </is>
+      </c>
+      <c r="F455" t="inlineStr">
+        <is>
+          <t>Data Staged</t>
+        </is>
+      </c>
+      <c r="G455" t="inlineStr"/>
+      <c r="H455" t="inlineStr"/>
+      <c r="I455" t="inlineStr"/>
+      <c r="J455" t="inlineStr"/>
+      <c r="K455" t="inlineStr"/>
+      <c r="L455" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M455" t="inlineStr"/>
+      <c r="N455" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O455" t="inlineStr"/>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>AN0130</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr"/>
+      <c r="C456" t="inlineStr"/>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>collection</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>T1114.001</t>
+        </is>
+      </c>
+      <c r="F456" t="inlineStr">
+        <is>
+          <t>Local Email Collection</t>
+        </is>
+      </c>
+      <c r="G456" t="inlineStr"/>
+      <c r="H456" t="inlineStr"/>
+      <c r="I456" t="inlineStr"/>
+      <c r="J456" t="inlineStr"/>
+      <c r="K456" t="inlineStr"/>
+      <c r="L456" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M456" t="inlineStr"/>
+      <c r="N456" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O456" t="inlineStr"/>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>AN0531</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr"/>
+      <c r="C457" t="inlineStr"/>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>collection</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>T1119</t>
+        </is>
+      </c>
+      <c r="F457" t="inlineStr">
+        <is>
+          <t>Automated Collection</t>
+        </is>
+      </c>
+      <c r="G457" t="inlineStr"/>
+      <c r="H457" t="inlineStr"/>
+      <c r="I457" t="inlineStr"/>
+      <c r="J457" t="inlineStr"/>
+      <c r="K457" t="inlineStr"/>
+      <c r="L457" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M457" t="inlineStr"/>
+      <c r="N457" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O457" t="inlineStr"/>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>AN0677</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr"/>
+      <c r="C458" t="inlineStr"/>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>collection</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>T1213.006</t>
+        </is>
+      </c>
+      <c r="F458" t="inlineStr">
+        <is>
+          <t>Databases</t>
+        </is>
+      </c>
+      <c r="G458" t="inlineStr"/>
+      <c r="H458" t="inlineStr"/>
+      <c r="I458" t="inlineStr"/>
+      <c r="J458" t="inlineStr"/>
+      <c r="K458" t="inlineStr"/>
+      <c r="L458" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M458" t="inlineStr"/>
+      <c r="N458" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O458" t="inlineStr"/>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>AN0724</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr"/>
+      <c r="C459" t="inlineStr"/>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>collection</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>T1074.001</t>
+        </is>
+      </c>
+      <c r="F459" t="inlineStr">
+        <is>
+          <t>Local Data Staging</t>
+        </is>
+      </c>
+      <c r="G459" t="inlineStr"/>
+      <c r="H459" t="inlineStr"/>
+      <c r="I459" t="inlineStr"/>
+      <c r="J459" t="inlineStr"/>
+      <c r="K459" t="inlineStr"/>
+      <c r="L459" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M459" t="inlineStr"/>
+      <c r="N459" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O459" t="inlineStr"/>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>AN0006</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr"/>
+      <c r="C460" t="inlineStr"/>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>persistence</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>T1136.002</t>
+        </is>
+      </c>
+      <c r="F460" t="inlineStr">
+        <is>
+          <t>Domain Account Creation</t>
+        </is>
+      </c>
+      <c r="G460" t="inlineStr"/>
+      <c r="H460" t="inlineStr"/>
+      <c r="I460" t="inlineStr"/>
+      <c r="J460" t="inlineStr"/>
+      <c r="K460" t="inlineStr"/>
+      <c r="L460" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M460" t="inlineStr"/>
+      <c r="N460" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O460" t="inlineStr"/>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>AN0045</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr"/>
+      <c r="C461" t="inlineStr"/>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>persistence</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>T1668</t>
+        </is>
+      </c>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>Exclusive Control</t>
+        </is>
+      </c>
+      <c r="G461" t="inlineStr"/>
+      <c r="H461" t="inlineStr"/>
+      <c r="I461" t="inlineStr"/>
+      <c r="J461" t="inlineStr"/>
+      <c r="K461" t="inlineStr"/>
+      <c r="L461" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M461" t="inlineStr"/>
+      <c r="N461" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O461" t="inlineStr"/>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>AN0137</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr"/>
+      <c r="C462" t="inlineStr"/>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>persistence</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>T1137.006</t>
+        </is>
+      </c>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>Add-ins</t>
+        </is>
+      </c>
+      <c r="G462" t="inlineStr"/>
+      <c r="H462" t="inlineStr"/>
+      <c r="I462" t="inlineStr"/>
+      <c r="J462" t="inlineStr"/>
+      <c r="K462" t="inlineStr"/>
+      <c r="L462" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M462" t="inlineStr"/>
+      <c r="N462" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O462" t="inlineStr"/>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>AN0184</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr"/>
+      <c r="C463" t="inlineStr"/>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>persistence</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>T1505.004</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>IIS Components</t>
+        </is>
+      </c>
+      <c r="G463" t="inlineStr"/>
+      <c r="H463" t="inlineStr"/>
+      <c r="I463" t="inlineStr"/>
+      <c r="J463" t="inlineStr"/>
+      <c r="K463" t="inlineStr"/>
+      <c r="L463" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M463" t="inlineStr"/>
+      <c r="N463" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O463" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refactor privilege escalation rules for multi-source log support
</commit_message>
<xml_diff>
--- a/ocsf_mapped_new_sprint.xlsx
+++ b/ocsf_mapped_new_sprint.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O463"/>
+  <dimension ref="A1:O474"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31967,6 +31967,457 @@
       </c>
       <c r="O463" t="inlineStr"/>
     </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>AN0024</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr"/>
+      <c r="C464" t="inlineStr"/>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>privilege-escalation</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>T1546</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>Windows Management Instrumentation Event Subscription</t>
+        </is>
+      </c>
+      <c r="G464" t="inlineStr"/>
+      <c r="H464" t="inlineStr"/>
+      <c r="I464" t="inlineStr"/>
+      <c r="J464" t="inlineStr"/>
+      <c r="K464" t="inlineStr"/>
+      <c r="L464" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M464" t="inlineStr"/>
+      <c r="N464" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O464" t="inlineStr"/>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>AN0051</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr"/>
+      <c r="C465" t="inlineStr"/>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>privilege-escalation</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>T1546.011</t>
+        </is>
+      </c>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>Application Shimming</t>
+        </is>
+      </c>
+      <c r="G465" t="inlineStr"/>
+      <c r="H465" t="inlineStr"/>
+      <c r="I465" t="inlineStr"/>
+      <c r="J465" t="inlineStr"/>
+      <c r="K465" t="inlineStr"/>
+      <c r="L465" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M465" t="inlineStr"/>
+      <c r="N465" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O465" t="inlineStr"/>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>AN0074</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr"/>
+      <c r="C466" t="inlineStr"/>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>privilege-escalation</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>T1547.012</t>
+        </is>
+      </c>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t>Print Processors</t>
+        </is>
+      </c>
+      <c r="G466" t="inlineStr"/>
+      <c r="H466" t="inlineStr"/>
+      <c r="I466" t="inlineStr"/>
+      <c r="J466" t="inlineStr"/>
+      <c r="K466" t="inlineStr"/>
+      <c r="L466" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M466" t="inlineStr"/>
+      <c r="N466" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O466" t="inlineStr"/>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>AN0094</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr"/>
+      <c r="C467" t="inlineStr"/>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>privilege-escalation</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>T1546.008</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>Accessibility Features</t>
+        </is>
+      </c>
+      <c r="G467" t="inlineStr"/>
+      <c r="H467" t="inlineStr"/>
+      <c r="I467" t="inlineStr"/>
+      <c r="J467" t="inlineStr"/>
+      <c r="K467" t="inlineStr"/>
+      <c r="L467" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M467" t="inlineStr"/>
+      <c r="N467" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O467" t="inlineStr"/>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>AN0170</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr"/>
+      <c r="C468" t="inlineStr"/>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>privilege-escalation</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>T1546.001</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>Change Default File Association</t>
+        </is>
+      </c>
+      <c r="G468" t="inlineStr"/>
+      <c r="H468" t="inlineStr"/>
+      <c r="I468" t="inlineStr"/>
+      <c r="J468" t="inlineStr"/>
+      <c r="K468" t="inlineStr"/>
+      <c r="L468" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M468" t="inlineStr"/>
+      <c r="N468" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O468" t="inlineStr"/>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>AN0590</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr"/>
+      <c r="C469" t="inlineStr"/>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>privilege-escalation</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>T1078.002</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>Domain Accounts</t>
+        </is>
+      </c>
+      <c r="G469" t="inlineStr"/>
+      <c r="H469" t="inlineStr"/>
+      <c r="I469" t="inlineStr"/>
+      <c r="J469" t="inlineStr"/>
+      <c r="K469" t="inlineStr"/>
+      <c r="L469" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M469" t="inlineStr"/>
+      <c r="N469" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O469" t="inlineStr"/>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>AN0975</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr"/>
+      <c r="C470" t="inlineStr"/>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>privilege-escalation</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>T1548</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>Abuse Elevation Control Mechanism</t>
+        </is>
+      </c>
+      <c r="G470" t="inlineStr"/>
+      <c r="H470" t="inlineStr"/>
+      <c r="I470" t="inlineStr"/>
+      <c r="J470" t="inlineStr"/>
+      <c r="K470" t="inlineStr"/>
+      <c r="L470" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M470" t="inlineStr"/>
+      <c r="N470" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O470" t="inlineStr"/>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>AN1094</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr"/>
+      <c r="C471" t="inlineStr"/>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>privilege-escalation</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>T1548.002</t>
+        </is>
+      </c>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t>Bypass User Account Control</t>
+        </is>
+      </c>
+      <c r="G471" t="inlineStr"/>
+      <c r="H471" t="inlineStr"/>
+      <c r="I471" t="inlineStr"/>
+      <c r="J471" t="inlineStr"/>
+      <c r="K471" t="inlineStr"/>
+      <c r="L471" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M471" t="inlineStr"/>
+      <c r="N471" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O471" t="inlineStr"/>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>AN1137</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr"/>
+      <c r="C472" t="inlineStr"/>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>privilege-escalation</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>T1078.003</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>Local Accounts</t>
+        </is>
+      </c>
+      <c r="G472" t="inlineStr"/>
+      <c r="H472" t="inlineStr"/>
+      <c r="I472" t="inlineStr"/>
+      <c r="J472" t="inlineStr"/>
+      <c r="K472" t="inlineStr"/>
+      <c r="L472" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M472" t="inlineStr"/>
+      <c r="N472" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O472" t="inlineStr"/>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>AN1283</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr"/>
+      <c r="C473" t="inlineStr"/>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>privilege-escalation</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>T1078.001</t>
+        </is>
+      </c>
+      <c r="F473" t="inlineStr">
+        <is>
+          <t>Default Accounts</t>
+        </is>
+      </c>
+      <c r="G473" t="inlineStr"/>
+      <c r="H473" t="inlineStr"/>
+      <c r="I473" t="inlineStr"/>
+      <c r="J473" t="inlineStr"/>
+      <c r="K473" t="inlineStr"/>
+      <c r="L473" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M473" t="inlineStr"/>
+      <c r="N473" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O473" t="inlineStr"/>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>AN1543</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr"/>
+      <c r="C474" t="inlineStr"/>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>privilege-escalation</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>T1078</t>
+        </is>
+      </c>
+      <c r="F474" t="inlineStr">
+        <is>
+          <t>Valid Accounts</t>
+        </is>
+      </c>
+      <c r="G474" t="inlineStr"/>
+      <c r="H474" t="inlineStr"/>
+      <c r="I474" t="inlineStr"/>
+      <c r="J474" t="inlineStr"/>
+      <c r="K474" t="inlineStr"/>
+      <c r="L474" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M474" t="inlineStr"/>
+      <c r="N474" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O474" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Commit all new sprint detection rules, logs summaries, and UUID fixes
</commit_message>
<xml_diff>
--- a/ocsf_mapped_new_sprint.xlsx
+++ b/ocsf_mapped_new_sprint.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O486"/>
+  <dimension ref="A1:O560"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -32222,6 +32222,2799 @@
         </is>
       </c>
     </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>AN2076</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>T1007</t>
+        </is>
+      </c>
+      <c r="F487" t="inlineStr">
+        <is>
+          <t>System Service Enumeration</t>
+        </is>
+      </c>
+      <c r="G487" t="inlineStr">
+        <is>
+          <t>DET0933</t>
+        </is>
+      </c>
+      <c r="J487" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1 (process_creation)</t>
+        </is>
+      </c>
+      <c r="L487" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N487" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>AN2077</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>T1012</t>
+        </is>
+      </c>
+      <c r="F488" t="inlineStr">
+        <is>
+          <t>Registry Query for Sensitive Configurations</t>
+        </is>
+      </c>
+      <c r="G488" t="inlineStr">
+        <is>
+          <t>DET0934</t>
+        </is>
+      </c>
+      <c r="J488" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1 (process_creation)</t>
+        </is>
+      </c>
+      <c r="L488" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N488" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>AN2078</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>T1016</t>
+        </is>
+      </c>
+      <c r="F489" t="inlineStr">
+        <is>
+          <t>System Network Configuration Enumeration</t>
+        </is>
+      </c>
+      <c r="G489" t="inlineStr">
+        <is>
+          <t>DET0935</t>
+        </is>
+      </c>
+      <c r="J489" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1 (process_creation)</t>
+        </is>
+      </c>
+      <c r="L489" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N489" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>AN2079</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>T1018</t>
+        </is>
+      </c>
+      <c r="F490" t="inlineStr">
+        <is>
+          <t>Remote System Discovery via Native Tools</t>
+        </is>
+      </c>
+      <c r="G490" t="inlineStr">
+        <is>
+          <t>DET0936</t>
+        </is>
+      </c>
+      <c r="J490" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1 (process_creation)</t>
+        </is>
+      </c>
+      <c r="L490" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N490" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>AN2080</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>T1046</t>
+        </is>
+      </c>
+      <c r="F491" t="inlineStr">
+        <is>
+          <t>Local Network Service Port Discovery</t>
+        </is>
+      </c>
+      <c r="G491" t="inlineStr">
+        <is>
+          <t>DET0937</t>
+        </is>
+      </c>
+      <c r="J491" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1 (process_creation)</t>
+        </is>
+      </c>
+      <c r="L491" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N491" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>AN2081</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>T1049</t>
+        </is>
+      </c>
+      <c r="F492" t="inlineStr">
+        <is>
+          <t>SMB Share and Session Discovery</t>
+        </is>
+      </c>
+      <c r="G492" t="inlineStr">
+        <is>
+          <t>DET0938</t>
+        </is>
+      </c>
+      <c r="J492" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1 (process_creation)</t>
+        </is>
+      </c>
+      <c r="L492" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N492" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>AN2082</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>T1069</t>
+        </is>
+      </c>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>Local and Domain Group Discovery</t>
+        </is>
+      </c>
+      <c r="G493" t="inlineStr">
+        <is>
+          <t>DET0939</t>
+        </is>
+      </c>
+      <c r="J493" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1 (process_creation)</t>
+        </is>
+      </c>
+      <c r="L493" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N493" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>AN2083</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>T1082</t>
+        </is>
+      </c>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t>System and Hardware Information Enumeration</t>
+        </is>
+      </c>
+      <c r="G494" t="inlineStr">
+        <is>
+          <t>DET0940</t>
+        </is>
+      </c>
+      <c r="J494" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1 (process_creation)</t>
+        </is>
+      </c>
+      <c r="L494" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N494" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>AN2084</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>T1083</t>
+        </is>
+      </c>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>Recursive Directory Enumeration</t>
+        </is>
+      </c>
+      <c r="G495" t="inlineStr">
+        <is>
+          <t>DET0941</t>
+        </is>
+      </c>
+      <c r="J495" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1 (process_creation)</t>
+        </is>
+      </c>
+      <c r="L495" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N495" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>AN2085</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>T1087</t>
+        </is>
+      </c>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>Local and Domain Account Enumeration</t>
+        </is>
+      </c>
+      <c r="G496" t="inlineStr">
+        <is>
+          <t>DET0942</t>
+        </is>
+      </c>
+      <c r="J496" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1 (process_creation)</t>
+        </is>
+      </c>
+      <c r="L496" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N496" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>AN2086</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>T1120</t>
+        </is>
+      </c>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>Peripheral Device Discovery via PowerShell or WMI</t>
+        </is>
+      </c>
+      <c r="G497" t="inlineStr">
+        <is>
+          <t>DET0943</t>
+        </is>
+      </c>
+      <c r="J497" t="inlineStr">
+        <is>
+          <t>Sysmon Event ID 1 / PowerShell Event ID 4104</t>
+        </is>
+      </c>
+      <c r="L497" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N497" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>AN2087</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>T1135</t>
+        </is>
+      </c>
+      <c r="F498" t="inlineStr">
+        <is>
+          <t>Network Share Enumeration via Native Tools</t>
+        </is>
+      </c>
+      <c r="G498" t="inlineStr">
+        <is>
+          <t>DET0944</t>
+        </is>
+      </c>
+      <c r="L498" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N498" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>AN2088</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>T1614</t>
+        </is>
+      </c>
+      <c r="F499" t="inlineStr">
+        <is>
+          <t>System Locale and Keyboard Layout Discovery</t>
+        </is>
+      </c>
+      <c r="G499" t="inlineStr">
+        <is>
+          <t>DET0945</t>
+        </is>
+      </c>
+      <c r="L499" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N499" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>AN2089</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>T1124</t>
+        </is>
+      </c>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>System Time and Timezone Discovery</t>
+        </is>
+      </c>
+      <c r="G500" t="inlineStr">
+        <is>
+          <t>DET0946</t>
+        </is>
+      </c>
+      <c r="L500" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N500" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>AN2090</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>T1615</t>
+        </is>
+      </c>
+      <c r="F501" t="inlineStr">
+        <is>
+          <t>Group Policy Enumeration</t>
+        </is>
+      </c>
+      <c r="G501" t="inlineStr">
+        <is>
+          <t>DET0947</t>
+        </is>
+      </c>
+      <c r="L501" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N501" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>AN2091</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>T1654</t>
+        </is>
+      </c>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>Windows Event Log Enumeration</t>
+        </is>
+      </c>
+      <c r="G502" t="inlineStr">
+        <is>
+          <t>DET0948</t>
+        </is>
+      </c>
+      <c r="L502" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N502" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>AN2092</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>T1652</t>
+        </is>
+      </c>
+      <c r="F503" t="inlineStr">
+        <is>
+          <t>Device Driver Enumeration</t>
+        </is>
+      </c>
+      <c r="G503" t="inlineStr">
+        <is>
+          <t>DET0949</t>
+        </is>
+      </c>
+      <c r="L503" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N503" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>AN2093</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="E504" t="inlineStr">
+        <is>
+          <t>T1040</t>
+        </is>
+      </c>
+      <c r="F504" t="inlineStr">
+        <is>
+          <t>Network Packet Capture Tool Execution</t>
+        </is>
+      </c>
+      <c r="G504" t="inlineStr">
+        <is>
+          <t>DET0950</t>
+        </is>
+      </c>
+      <c r="L504" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N504" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>AN2094</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="E505" t="inlineStr">
+        <is>
+          <t>T1497</t>
+        </is>
+      </c>
+      <c r="F505" t="inlineStr">
+        <is>
+          <t>VM and Sandbox Detection Artifact Queries</t>
+        </is>
+      </c>
+      <c r="G505" t="inlineStr">
+        <is>
+          <t>DET0951</t>
+        </is>
+      </c>
+      <c r="L505" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N505" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>AN2095</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="E506" t="inlineStr">
+        <is>
+          <t>T1673</t>
+        </is>
+      </c>
+      <c r="F506" t="inlineStr">
+        <is>
+          <t>Virtual Machine Infrastructure Enumeration</t>
+        </is>
+      </c>
+      <c r="G506" t="inlineStr">
+        <is>
+          <t>DET0952</t>
+        </is>
+      </c>
+      <c r="L506" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N506" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>AN2096</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>T1680</t>
+        </is>
+      </c>
+      <c r="F507" t="inlineStr">
+        <is>
+          <t>Local Storage Device Enumeration</t>
+        </is>
+      </c>
+      <c r="G507" t="inlineStr">
+        <is>
+          <t>DET0953</t>
+        </is>
+      </c>
+      <c r="L507" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N507" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>AN2097</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="E508" t="inlineStr">
+        <is>
+          <t>T1622</t>
+        </is>
+      </c>
+      <c r="F508" t="inlineStr">
+        <is>
+          <t>Debugger Presence Check via Registry or Process Query</t>
+        </is>
+      </c>
+      <c r="G508" t="inlineStr">
+        <is>
+          <t>DET0954</t>
+        </is>
+      </c>
+      <c r="L508" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N508" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>AN2098</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E509" t="inlineStr">
+        <is>
+          <t>T1197</t>
+        </is>
+      </c>
+      <c r="G509" t="inlineStr">
+        <is>
+          <t>DET0955</t>
+        </is>
+      </c>
+      <c r="H509" t="inlineStr">
+        <is>
+          <t>BITS Job Transfer or Notification Command Abuse</t>
+        </is>
+      </c>
+      <c r="L509" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N509" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>AN2099</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E510" t="inlineStr">
+        <is>
+          <t>T1140</t>
+        </is>
+      </c>
+      <c r="G510" t="inlineStr">
+        <is>
+          <t>DET0956</t>
+        </is>
+      </c>
+      <c r="H510" t="inlineStr">
+        <is>
+          <t>File Decode or Deobfuscation via LOLBins</t>
+        </is>
+      </c>
+      <c r="L510" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N510" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>AN2100</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E511" t="inlineStr">
+        <is>
+          <t>T1202</t>
+        </is>
+      </c>
+      <c r="G511" t="inlineStr">
+        <is>
+          <t>DET0957</t>
+        </is>
+      </c>
+      <c r="H511" t="inlineStr">
+        <is>
+          <t>Indirect Command Execution via Trusted Windows Utilities</t>
+        </is>
+      </c>
+      <c r="L511" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N511" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>AN2101</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E512" t="inlineStr">
+        <is>
+          <t>T1216</t>
+        </is>
+      </c>
+      <c r="G512" t="inlineStr">
+        <is>
+          <t>DET0958</t>
+        </is>
+      </c>
+      <c r="H512" t="inlineStr">
+        <is>
+          <t>Microsoft-Signed Script Proxy Execution</t>
+        </is>
+      </c>
+      <c r="L512" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N512" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>AN2102</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E513" t="inlineStr">
+        <is>
+          <t>T1220</t>
+        </is>
+      </c>
+      <c r="G513" t="inlineStr">
+        <is>
+          <t>DET0959</t>
+        </is>
+      </c>
+      <c r="H513" t="inlineStr">
+        <is>
+          <t>XSL Script Execution via WMIC or MSXSL</t>
+        </is>
+      </c>
+      <c r="L513" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N513" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>AN2103</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>Credential Access</t>
+        </is>
+      </c>
+      <c r="E514" t="inlineStr">
+        <is>
+          <t>T1552</t>
+        </is>
+      </c>
+      <c r="G514" t="inlineStr">
+        <is>
+          <t>DET0960</t>
+        </is>
+      </c>
+      <c r="H514" t="inlineStr">
+        <is>
+          <t>Credential String Search in Files and Registry</t>
+        </is>
+      </c>
+      <c r="L514" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N514" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>AN2104</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>Credential Access</t>
+        </is>
+      </c>
+      <c r="E515" t="inlineStr">
+        <is>
+          <t>T1187</t>
+        </is>
+      </c>
+      <c r="G515" t="inlineStr">
+        <is>
+          <t>DET0961</t>
+        </is>
+      </c>
+      <c r="H515" t="inlineStr">
+        <is>
+          <t>Forced Authentication via UNC Path or SCF File Creation</t>
+        </is>
+      </c>
+      <c r="L515" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N515" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>AN2105</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E516" t="inlineStr">
+        <is>
+          <t>T1036</t>
+        </is>
+      </c>
+      <c r="G516" t="inlineStr">
+        <is>
+          <t>DET0962</t>
+        </is>
+      </c>
+      <c r="H516" t="inlineStr">
+        <is>
+          <t>System Binary Name Used from Non-Standard Path</t>
+        </is>
+      </c>
+      <c r="L516" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N516" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>AN2106</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E517" t="inlineStr">
+        <is>
+          <t>T1027</t>
+        </is>
+      </c>
+      <c r="G517" t="inlineStr">
+        <is>
+          <t>DET0963</t>
+        </is>
+      </c>
+      <c r="H517" t="inlineStr">
+        <is>
+          <t>PowerShell Encoded Command or Heavy Obfuscation Execution</t>
+        </is>
+      </c>
+      <c r="L517" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N517" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>AN2107</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>Credential Access</t>
+        </is>
+      </c>
+      <c r="E518" t="inlineStr">
+        <is>
+          <t>T1539</t>
+        </is>
+      </c>
+      <c r="G518" t="inlineStr">
+        <is>
+          <t>DET0964</t>
+        </is>
+      </c>
+      <c r="H518" t="inlineStr">
+        <is>
+          <t>Browser Cookie Database Access by Non-Browser Process</t>
+        </is>
+      </c>
+      <c r="L518" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N518" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>AN2108</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E519" t="inlineStr">
+        <is>
+          <t>T1001</t>
+        </is>
+      </c>
+      <c r="G519" t="inlineStr">
+        <is>
+          <t>DET0965</t>
+        </is>
+      </c>
+      <c r="H519" t="inlineStr">
+        <is>
+          <t>Steganography or Data Obfuscation Utility Execution</t>
+        </is>
+      </c>
+      <c r="L519" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N519" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>AN2109</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E520" t="inlineStr">
+        <is>
+          <t>T1006</t>
+        </is>
+      </c>
+      <c r="G520" t="inlineStr">
+        <is>
+          <t>DET0966</t>
+        </is>
+      </c>
+      <c r="H520" t="inlineStr">
+        <is>
+          <t>Direct Volume Access Command Line Detection</t>
+        </is>
+      </c>
+      <c r="L520" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N520" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>AN2110</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>Command and Control</t>
+        </is>
+      </c>
+      <c r="E521" t="inlineStr">
+        <is>
+          <t>T1008</t>
+        </is>
+      </c>
+      <c r="G521" t="inlineStr">
+        <is>
+          <t>DET0967</t>
+        </is>
+      </c>
+      <c r="H521" t="inlineStr">
+        <is>
+          <t>Redundant Fallback Channel Proxy Execution</t>
+        </is>
+      </c>
+      <c r="L521" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N521" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>AN2111</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E522" t="inlineStr">
+        <is>
+          <t>T1014</t>
+        </is>
+      </c>
+      <c r="G522" t="inlineStr">
+        <is>
+          <t>DET0968</t>
+        </is>
+      </c>
+      <c r="H522" t="inlineStr">
+        <is>
+          <t>Rootkit Installation or Kernel Driver Bypass Tool Execution</t>
+        </is>
+      </c>
+      <c r="L522" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N522" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>AN2112</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>Persistence</t>
+        </is>
+      </c>
+      <c r="E523" t="inlineStr">
+        <is>
+          <t>T1037</t>
+        </is>
+      </c>
+      <c r="G523" t="inlineStr">
+        <is>
+          <t>DET0969</t>
+        </is>
+      </c>
+      <c r="H523" t="inlineStr">
+        <is>
+          <t>User Logon Initialization Script Registry Modification</t>
+        </is>
+      </c>
+      <c r="L523" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N523" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>AN2113</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>Command and Control</t>
+        </is>
+      </c>
+      <c r="E524" t="inlineStr">
+        <is>
+          <t>T1092</t>
+        </is>
+      </c>
+      <c r="G524" t="inlineStr">
+        <is>
+          <t>DET0970</t>
+        </is>
+      </c>
+      <c r="H524" t="inlineStr">
+        <is>
+          <t>Script or Binary Execution from Removable Media Path</t>
+        </is>
+      </c>
+      <c r="L524" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N524" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>AN2114</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>Persistence</t>
+        </is>
+      </c>
+      <c r="E525" t="inlineStr">
+        <is>
+          <t>T1098</t>
+        </is>
+      </c>
+      <c r="G525" t="inlineStr">
+        <is>
+          <t>DET0971</t>
+        </is>
+      </c>
+      <c r="H525" t="inlineStr">
+        <is>
+          <t>Privileged Account or Group Membership Manipulation</t>
+        </is>
+      </c>
+      <c r="L525" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N525" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>AN2115</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>Credential Access</t>
+        </is>
+      </c>
+      <c r="E526" t="inlineStr">
+        <is>
+          <t>T1111</t>
+        </is>
+      </c>
+      <c r="G526" t="inlineStr">
+        <is>
+          <t>DET0972</t>
+        </is>
+      </c>
+      <c r="H526" t="inlineStr">
+        <is>
+          <t>Custom Security Support Provider or LSA Package Registration</t>
+        </is>
+      </c>
+      <c r="L526" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N526" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>AN2116</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>Command and Control</t>
+        </is>
+      </c>
+      <c r="E527" t="inlineStr">
+        <is>
+          <t>T1132</t>
+        </is>
+      </c>
+      <c r="G527" t="inlineStr">
+        <is>
+          <t>DET0973</t>
+        </is>
+      </c>
+      <c r="H527" t="inlineStr">
+        <is>
+          <t>Process Command Line Data Encoding or Decoding Activity</t>
+        </is>
+      </c>
+      <c r="L527" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N527" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>AN2117</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E528" t="inlineStr">
+        <is>
+          <t>T1211</t>
+        </is>
+      </c>
+      <c r="G528" t="inlineStr">
+        <is>
+          <t>DET0974</t>
+        </is>
+      </c>
+      <c r="H528" t="inlineStr">
+        <is>
+          <t>Anomalous Handle Access to System Process for Exploitation or Stealth</t>
+        </is>
+      </c>
+      <c r="L528" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N528" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>AN2118</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>Credential Access</t>
+        </is>
+      </c>
+      <c r="E529" t="inlineStr">
+        <is>
+          <t>T1212</t>
+        </is>
+      </c>
+      <c r="G529" t="inlineStr">
+        <is>
+          <t>DET0975</t>
+        </is>
+      </c>
+      <c r="H529" t="inlineStr">
+        <is>
+          <t>Print Spooler Service Spawning Suspicious Child Process</t>
+        </is>
+      </c>
+      <c r="L529" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N529" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>AN2108</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E530" t="inlineStr">
+        <is>
+          <t>T1001</t>
+        </is>
+      </c>
+      <c r="G530" t="inlineStr">
+        <is>
+          <t>DET0965</t>
+        </is>
+      </c>
+      <c r="H530" t="inlineStr">
+        <is>
+          <t>Steganography or Data Obfuscation Utility Execution</t>
+        </is>
+      </c>
+      <c r="L530" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N530" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>AN2109</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E531" t="inlineStr">
+        <is>
+          <t>T1006</t>
+        </is>
+      </c>
+      <c r="G531" t="inlineStr">
+        <is>
+          <t>DET0966</t>
+        </is>
+      </c>
+      <c r="H531" t="inlineStr">
+        <is>
+          <t>Direct Volume Access Command Line Detection</t>
+        </is>
+      </c>
+      <c r="L531" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N531" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>AN2110</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>Command and Control</t>
+        </is>
+      </c>
+      <c r="E532" t="inlineStr">
+        <is>
+          <t>T1008</t>
+        </is>
+      </c>
+      <c r="G532" t="inlineStr">
+        <is>
+          <t>DET0967</t>
+        </is>
+      </c>
+      <c r="H532" t="inlineStr">
+        <is>
+          <t>Redundant Fallback Channel Proxy Execution</t>
+        </is>
+      </c>
+      <c r="L532" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N532" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>AN2111</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E533" t="inlineStr">
+        <is>
+          <t>T1014</t>
+        </is>
+      </c>
+      <c r="G533" t="inlineStr">
+        <is>
+          <t>DET0968</t>
+        </is>
+      </c>
+      <c r="H533" t="inlineStr">
+        <is>
+          <t>Rootkit Installation or Kernel Driver Bypass Tool Execution</t>
+        </is>
+      </c>
+      <c r="L533" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N533" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>AN2112</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>Persistence</t>
+        </is>
+      </c>
+      <c r="E534" t="inlineStr">
+        <is>
+          <t>T1037</t>
+        </is>
+      </c>
+      <c r="G534" t="inlineStr">
+        <is>
+          <t>DET0969</t>
+        </is>
+      </c>
+      <c r="H534" t="inlineStr">
+        <is>
+          <t>User Logon Initialization Script Registry Modification</t>
+        </is>
+      </c>
+      <c r="L534" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N534" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>AN2113</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>Command and Control</t>
+        </is>
+      </c>
+      <c r="E535" t="inlineStr">
+        <is>
+          <t>T1092</t>
+        </is>
+      </c>
+      <c r="G535" t="inlineStr">
+        <is>
+          <t>DET0970</t>
+        </is>
+      </c>
+      <c r="H535" t="inlineStr">
+        <is>
+          <t>Script or Binary Execution from Removable Media Path</t>
+        </is>
+      </c>
+      <c r="L535" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N535" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>AN2114</t>
+        </is>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>Persistence</t>
+        </is>
+      </c>
+      <c r="E536" t="inlineStr">
+        <is>
+          <t>T1098</t>
+        </is>
+      </c>
+      <c r="G536" t="inlineStr">
+        <is>
+          <t>DET0971</t>
+        </is>
+      </c>
+      <c r="H536" t="inlineStr">
+        <is>
+          <t>Privileged Account or Group Membership Manipulation</t>
+        </is>
+      </c>
+      <c r="L536" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N536" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>AN2115</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>Credential Access</t>
+        </is>
+      </c>
+      <c r="E537" t="inlineStr">
+        <is>
+          <t>T1111</t>
+        </is>
+      </c>
+      <c r="G537" t="inlineStr">
+        <is>
+          <t>DET0972</t>
+        </is>
+      </c>
+      <c r="H537" t="inlineStr">
+        <is>
+          <t>Custom Security Support Provider or LSA Package Registration</t>
+        </is>
+      </c>
+      <c r="L537" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N537" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>AN2116</t>
+        </is>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>Command and Control</t>
+        </is>
+      </c>
+      <c r="E538" t="inlineStr">
+        <is>
+          <t>T1132</t>
+        </is>
+      </c>
+      <c r="G538" t="inlineStr">
+        <is>
+          <t>DET0973</t>
+        </is>
+      </c>
+      <c r="H538" t="inlineStr">
+        <is>
+          <t>Process Command Line Data Encoding or Decoding Activity</t>
+        </is>
+      </c>
+      <c r="L538" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N538" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>AN2117</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E539" t="inlineStr">
+        <is>
+          <t>T1211</t>
+        </is>
+      </c>
+      <c r="G539" t="inlineStr">
+        <is>
+          <t>DET0974</t>
+        </is>
+      </c>
+      <c r="H539" t="inlineStr">
+        <is>
+          <t>Anomalous Handle Access to System Process for Exploitation or Stealth</t>
+        </is>
+      </c>
+      <c r="L539" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N539" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>AN2118</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>Credential Access</t>
+        </is>
+      </c>
+      <c r="E540" t="inlineStr">
+        <is>
+          <t>T1212</t>
+        </is>
+      </c>
+      <c r="G540" t="inlineStr">
+        <is>
+          <t>DET0975</t>
+        </is>
+      </c>
+      <c r="H540" t="inlineStr">
+        <is>
+          <t>Print Spooler Service Spawning Suspicious Child Process</t>
+        </is>
+      </c>
+      <c r="L540" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N540" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>AN2119</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E541" t="inlineStr">
+        <is>
+          <t>T1221</t>
+        </is>
+      </c>
+      <c r="G541" t="inlineStr">
+        <is>
+          <t>DET0976</t>
+        </is>
+      </c>
+      <c r="H541" t="inlineStr">
+        <is>
+          <t>Microsoft Office Application Spawning Script Interpreter</t>
+        </is>
+      </c>
+      <c r="L541" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N541" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>AN2120</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E542" t="inlineStr">
+        <is>
+          <t>T1480</t>
+        </is>
+      </c>
+      <c r="G542" t="inlineStr">
+        <is>
+          <t>DET0977</t>
+        </is>
+      </c>
+      <c r="H542" t="inlineStr">
+        <is>
+          <t>Execution Guardrails Target Discovery Query</t>
+        </is>
+      </c>
+      <c r="L542" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N542" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>AN2121</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>Persistence</t>
+        </is>
+      </c>
+      <c r="E543" t="inlineStr">
+        <is>
+          <t>T1542</t>
+        </is>
+      </c>
+      <c r="G543" t="inlineStr">
+        <is>
+          <t>DET0978</t>
+        </is>
+      </c>
+      <c r="H543" t="inlineStr">
+        <is>
+          <t>System Firmware or BIOS Flash Utility Execution</t>
+        </is>
+      </c>
+      <c r="L543" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N543" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>AN2122</t>
+        </is>
+      </c>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E544" t="inlineStr">
+        <is>
+          <t>T1620</t>
+        </is>
+      </c>
+      <c r="G544" t="inlineStr">
+        <is>
+          <t>DET0979</t>
+        </is>
+      </c>
+      <c r="H544" t="inlineStr">
+        <is>
+          <t>PowerShell Reflective Code Loading API Call</t>
+        </is>
+      </c>
+      <c r="L544" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N544" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>AN2123</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>Credential Access</t>
+        </is>
+      </c>
+      <c r="E545" t="inlineStr">
+        <is>
+          <t>T1649</t>
+        </is>
+      </c>
+      <c r="G545" t="inlineStr">
+        <is>
+          <t>DET0980</t>
+        </is>
+      </c>
+      <c r="H545" t="inlineStr">
+        <is>
+          <t>Authentication Certificate or Private Key Export Tool Execution</t>
+        </is>
+      </c>
+      <c r="L545" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N545" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>AN2124</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E546" t="inlineStr">
+        <is>
+          <t>T1665</t>
+        </is>
+      </c>
+      <c r="G546" t="inlineStr">
+        <is>
+          <t>DET0981</t>
+        </is>
+      </c>
+      <c r="H546" t="inlineStr">
+        <is>
+          <t>Network DNS Resolver or Interface Routing Hijack</t>
+        </is>
+      </c>
+      <c r="L546" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N546" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>AN2125</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>T1674</t>
+        </is>
+      </c>
+      <c r="G547" t="inlineStr">
+        <is>
+          <t>DET0982</t>
+        </is>
+      </c>
+      <c r="H547" t="inlineStr">
+        <is>
+          <t>Input Keystroke Automation or Injection Tool Execution</t>
+        </is>
+      </c>
+      <c r="L547" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N547" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>AN2126</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E548" t="inlineStr">
+        <is>
+          <t>T1678</t>
+        </is>
+      </c>
+      <c r="G548" t="inlineStr">
+        <is>
+          <t>DET0983</t>
+        </is>
+      </c>
+      <c r="H548" t="inlineStr">
+        <is>
+          <t>Artificial Execution Delay or Anti-Sandbox Sleep</t>
+        </is>
+      </c>
+      <c r="L548" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N548" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>AN2127</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>T1679</t>
+        </is>
+      </c>
+      <c r="G549" t="inlineStr">
+        <is>
+          <t>DET0984</t>
+        </is>
+      </c>
+      <c r="H549" t="inlineStr">
+        <is>
+          <t>Windows Defender Selective Exclusion Configuration</t>
+        </is>
+      </c>
+      <c r="L549" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N549" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>AN2128</t>
+        </is>
+      </c>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>Credential Access</t>
+        </is>
+      </c>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>T1684</t>
+        </is>
+      </c>
+      <c r="G550" t="inlineStr">
+        <is>
+          <t>DET0985</t>
+        </is>
+      </c>
+      <c r="H550" t="inlineStr">
+        <is>
+          <t>Social Engineering Script-Based Credential Dialog Prompt</t>
+        </is>
+      </c>
+      <c r="L550" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N550" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>AN2119</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>T1221</t>
+        </is>
+      </c>
+      <c r="G551" t="inlineStr">
+        <is>
+          <t>DET0976</t>
+        </is>
+      </c>
+      <c r="H551" t="inlineStr">
+        <is>
+          <t>Microsoft Office Application Spawning Script Interpreter</t>
+        </is>
+      </c>
+      <c r="L551" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N551" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>AN2120</t>
+        </is>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E552" t="inlineStr">
+        <is>
+          <t>T1480</t>
+        </is>
+      </c>
+      <c r="G552" t="inlineStr">
+        <is>
+          <t>DET0977</t>
+        </is>
+      </c>
+      <c r="H552" t="inlineStr">
+        <is>
+          <t>Execution Guardrails Target Discovery Query</t>
+        </is>
+      </c>
+      <c r="L552" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N552" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>AN2121</t>
+        </is>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>Persistence</t>
+        </is>
+      </c>
+      <c r="E553" t="inlineStr">
+        <is>
+          <t>T1542</t>
+        </is>
+      </c>
+      <c r="G553" t="inlineStr">
+        <is>
+          <t>DET0978</t>
+        </is>
+      </c>
+      <c r="H553" t="inlineStr">
+        <is>
+          <t>System Firmware or BIOS Flash Utility Execution</t>
+        </is>
+      </c>
+      <c r="L553" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N553" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>AN2122</t>
+        </is>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E554" t="inlineStr">
+        <is>
+          <t>T1620</t>
+        </is>
+      </c>
+      <c r="G554" t="inlineStr">
+        <is>
+          <t>DET0979</t>
+        </is>
+      </c>
+      <c r="H554" t="inlineStr">
+        <is>
+          <t>PowerShell Reflective Code Loading API Call</t>
+        </is>
+      </c>
+      <c r="L554" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N554" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>AN2123</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>Credential Access</t>
+        </is>
+      </c>
+      <c r="E555" t="inlineStr">
+        <is>
+          <t>T1649</t>
+        </is>
+      </c>
+      <c r="G555" t="inlineStr">
+        <is>
+          <t>DET0980</t>
+        </is>
+      </c>
+      <c r="H555" t="inlineStr">
+        <is>
+          <t>Authentication Certificate or Private Key Export Tool Execution</t>
+        </is>
+      </c>
+      <c r="L555" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N555" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>AN2124</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E556" t="inlineStr">
+        <is>
+          <t>T1665</t>
+        </is>
+      </c>
+      <c r="G556" t="inlineStr">
+        <is>
+          <t>DET0981</t>
+        </is>
+      </c>
+      <c r="H556" t="inlineStr">
+        <is>
+          <t>Network DNS Resolver or Interface Routing Hijack</t>
+        </is>
+      </c>
+      <c r="L556" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N556" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>AN2125</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>T1674</t>
+        </is>
+      </c>
+      <c r="G557" t="inlineStr">
+        <is>
+          <t>DET0982</t>
+        </is>
+      </c>
+      <c r="H557" t="inlineStr">
+        <is>
+          <t>Input Keystroke Automation or Injection Tool Execution</t>
+        </is>
+      </c>
+      <c r="L557" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N557" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>AN2126</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>T1678</t>
+        </is>
+      </c>
+      <c r="G558" t="inlineStr">
+        <is>
+          <t>DET0983</t>
+        </is>
+      </c>
+      <c r="H558" t="inlineStr">
+        <is>
+          <t>Artificial Execution Delay or Anti-Sandbox Sleep</t>
+        </is>
+      </c>
+      <c r="L558" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N558" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>AN2127</t>
+        </is>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>T1679</t>
+        </is>
+      </c>
+      <c r="G559" t="inlineStr">
+        <is>
+          <t>DET0984</t>
+        </is>
+      </c>
+      <c r="H559" t="inlineStr">
+        <is>
+          <t>Windows Defender Selective Exclusion Configuration</t>
+        </is>
+      </c>
+      <c r="L559" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N559" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>AN2128</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>Credential Access</t>
+        </is>
+      </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>T1684</t>
+        </is>
+      </c>
+      <c r="G560" t="inlineStr">
+        <is>
+          <t>DET0985</t>
+        </is>
+      </c>
+      <c r="H560" t="inlineStr">
+        <is>
+          <t>Social Engineering Script-Based Credential Dialog Prompt</t>
+        </is>
+      </c>
+      <c r="L560" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N560" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>